<commit_message>
paper: actualización diaria 2026-09-30
</commit_message>
<xml_diff>
--- a/millonary/paper_state/semanal/diario.xlsx
+++ b/millonary/paper_state/semanal/diario.xlsx
@@ -442,7 +442,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-29 17:40:34.148932+00:00</t>
+          <t>2026-09-30 04:18:19.127437+00:00</t>
         </is>
       </c>
     </row>
@@ -500,7 +500,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>{"n_pruebas": 75, "etapas": {"descartada (E1/E2)": 54, "E3 sombra": 21}, "adoptables": [], "top_forward": [], "ultima_actualizacion": "2026-09-29 17:40:34.148932+00:00"}</t>
+          <t>{"n_pruebas": 75, "etapas": {"descartada (E1/E2)": 54, "E3 sombra": 21}, "adoptables": [], "top_forward": [], "ultima_actualizacion": "2026-09-30 04:18:19.127437+00:00"}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
informe diario: corrige el punto de partida (inicio fuera de la rejilla de 4 h) y réplica de estado; panel: pestaña Marcador (ganadas/perdidas)
</commit_message>
<xml_diff>
--- a/millonary/paper_state/semanal/diario.xlsx
+++ b/millonary/paper_state/semanal/diario.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -442,7 +442,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-30 04:18:19.127437+00:00</t>
+          <t>2026-10-01 10:11:05.733781+00:00</t>
         </is>
       </c>
     </row>
@@ -453,54 +453,242 @@
         </is>
       </c>
       <c r="B3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>estado_comite</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>AVISO</t>
-        </is>
+          <t>equity_inicial</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>999.59048574632</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>decision</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Mantener el objetivo del núcleo: 0.62× de exposición.</t>
-        </is>
+          <t>equity_actual</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>999.537475038766</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>incubadora</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>{"certificadas": [], "forward": {"S01 Parabolic SAR + EMA200": {"retorno": 0.0, "caida_max": 0.0, "ops": 0, "dias": 0, "sharpe": null, "posicion_actual": 0.0}, "S02 Ichimoku": {"retorno": 0.0, "caida_max": 0.0, "ops": 0, "dias": 0, "sharpe": null, "posicion_actual": 0.0}, "S03 Bollinger + RSI (reversi\u00f3n)": {"retorno": 0.0, "caida_max": 0.0, "ops": 0, "dias": 0, "sharpe": null, "posicion_actual": 0.0}, "S04 Keltner ruptura": {"retorno": 0.0, "caida_max": 0.0, "ops": 0, "dias": 0, "sharpe": null, "posicion_actual": 0.0}, "S05 RSI(2) retroceso (largo)": {"retorno": 0.0, "caida_max": 0.0, "ops": 0, "dias": 0, "sharpe": null, "posicion_actual": 0.0}, "S06 Cruce SMA 7-25": {"retorno": 0.0, "caida_max": 0.0, "ops": 0, "dias": 0, "sharpe": null, "posicion_actual": -1.0}, "S07 SMA 7-25 + filtro 200 (largo)": {"retorno": 0.0, "caida_max": 0.0, "ops": 0, "dias": 0, "sharpe": null, "posicion_actual": 0.0}, "S08 Canal 20 por tercios": {"retorno": 0.0, "caida_max": 0.0, "ops": 0, "dias": 0, "sharpe": null, "posicion_actual": 0.0}, "S09 Donchian 20/10": {"retorno": 0.0, "caida_max": 0.0, "ops": 0, "dias": 0, "sharpe": null, "posicion_actual": -1.0}, "S10 MACD + EMA200": {"retorno": 0.0, "caida_max": 0.0, "ops": 0, "dias": 0, "sharpe": null, "posicion_actual": 0.0}, "S11 Supertrend 10/3": {"retorno": 0.0, "caida_max": 0.0, "ops": 0, "dias": 0, "sharpe": null, "posicion_actual": -1.0}, "S12 Expansi\u00f3n de volatilidad": {"retorno": 0.0, "caida_max": 0.0, "ops": 0, "dias": 0, "sharpe": null, "posicion_actual": 0.0}, "S13 Retroceso a EMA20": {"retorno": 0.0, "caida_max": 0.0, "ops": 0, "dias": 0, "sharpe": null, "posicion_actual": 0.0}, "S14 Momentum 90 d": {"retorno": 0.0, "caida_max": 0.0, "ops": 0, "dias": 0, "sharpe": null, "posicion_actual": 1.0}, "S15 RSI14 + EMA200": {"retorno": 0.0, "caida_max": 0.0, "ops": 0, "dias": 0, "sharpe": null, "posicion_actual": 0.0}}}</t>
-        </is>
+          <t>retorno_total</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>-5.303242508802875e-05</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>retorno_semana</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>-5.303242508802875e-05</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>caida_max</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0.003742184637251178</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>caida_actual</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0.003742184637251178</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>dias</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>velas</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>exposicion_actual</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0.5853090200318001</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>velas_semana</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>ordenes_total</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>ordenes_semana</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>comisiones_total</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0.29252689368</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>comisiones_semana</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>0.29252689368</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>posiciones</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>{"cerradas": 0, "ganan": 0, "pierden": 0, "abiertas": 1}</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>lotes</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>{"cerrados": 0, "ganan": 0, "pierden": 0, "abiertos": 1}</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>puertas</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>{"G1_replica": false, "G2_integridad": true, "G3_envolvente": true, "G4_no_anomalo": true, "G5_registro_cuadra": true}</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>posterior_sharpe</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>{"dias": 2, "estado": "insuficiente"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>estado_comite</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>decision</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Mantener el objetivo del núcleo: 0.62× de exposición.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>incubadora</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>{"certificadas": [], "forward": {"S01 Parabolic SAR + EMA200": {"retorno": -0.0007663354382617671, "caida_max": 0.006377236760283789, "ops": 1, "dias": 2, "sharpe": null, "posicion_actual": 1.0}, "S02 Ichimoku": {"retorno": 0.0, "caida_max": 0.0, "ops": 0, "dias": 2, "sharpe": null, "posicion_actual": 0.0}, "S03 Bollinger + RSI (reversi\u00f3n)": {"retorno": 0.0, "caida_max": 0.0, "ops": 0, "dias": 2, "sharpe": null, "posicion_actual": 0.0}, "S04 Keltner ruptura": {"retorno": 0.0, "caida_max": 0.0, "ops": 0, "dias": 2, "sharpe": null, "posicion_actual": 0.0}, "S05 RSI(2) retroceso (largo)": {"retorno": 0.0, "caida_max": 0.0, "ops": 0, "dias": 2, "sharpe": null, "posicion_actual": 0.0}, "S06 Cruce SMA 7-25": {"retorno": -0.0007555304832757015, "caida_max": 0.010057059455663264, "ops": 1, "dias": 2, "sharpe": null, "posicion_actual": -1.0}, "S07 SMA 7-25 + filtro 200 (largo)": {"retorno": 0.0, "caida_max": 0.0, "ops": 0, "dias": 2, "sharpe": null, "posicion_actual": 0.0}, "S08 Canal 20 por tercios": {"retorno": -0.008755142750290323, "caida_max": 0.008755142750290323, "ops": 1, "dias": 2, "sharpe": null, "posicion_actual": 0.0}, "S09 Donchian 20/10": {"retorno": -0.0007555304832757015, "caida_max": 0.010057059455663264, "ops": 1, "dias": 2, "sharpe": null, "posicion_actual": -1.0}, "S10 MACD + EMA200": {"retorno": -0.0045099301825412, "caida_max": 0.006377236760283789, "ops": 1, "dias": 2, "sharpe": null, "posicion_actual": 1.0}, "S11 Supertrend 10/3": {"retorno": -0.0007555304832757015, "caida_max": 0.010057059455663264, "ops": 1, "dias": 2, "sharpe": null, "posicion_actual": -1.0}, "S12 Expansi\u00f3n de volatilidad": {"retorno": -0.007077236284004473, "caida_max": 0.007077236284004473, "ops": 1, "dias": 2, "sharpe": null, "posicion_actual": 0.0}, "S13 Retroceso a EMA20": {"retorno": -0.0045099301825412, "caida_max": 0.006377236760283789, "ops": 1, "dias": 2, "sharpe": null, "posicion_actual": 1.0}, "S14 Momentum 90 d": {"retorno": -0.0007663354382617671, "caida_max": 0.006377236760283789, "ops": 1, "dias": 2, "sharpe": null, "posicion_actual": 1.0}, "S15 RSI14 + EMA200": {"retorno": 0.0, "caida_max": 0.0, "ops": 0, "dias": 2, "sharpe": null, "posicion_actual": 0.0}}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
           <t>mejoras</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>{"n_pruebas": 75, "etapas": {"descartada (E1/E2)": 54, "E3 sombra": 21}, "adoptables": [], "top_forward": [], "ultima_actualizacion": "2026-09-30 04:18:19.127437+00:00"}</t>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>{"n_pruebas": 75, "etapas": {"descartada (E1/E2)": 54, "E3 sombra": 21}, "adoptables": [], "top_forward": [], "ultima_actualizacion": "2026-10-01 10:11:05.733781+00:00"}</t>
         </is>
       </c>
     </row>
@@ -515,22 +703,287 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>info</t>
+          <t>bar</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>equity</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>units</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>price</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>expo</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>signal</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>target</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>funding</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>flags</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>sin datos todavía</t>
-        </is>
-      </c>
+          <t>2026-09-29 20:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>999.59048574632</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="D2" t="n">
+        <v>83562.39999999999</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.5851764380923165</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.6112786450001938</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-09-30 00:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>999.9666485963201</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="D3" t="n">
+        <v>83624.5</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.5853910236123392</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.6135457420193983</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.05853715</v>
+      </c>
+      <c r="I3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-09-30 04:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>997.48514859632</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="D4" t="n">
+        <v>83270</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.5843595775037391</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.614912747741446</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-09-30 08:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>997.408170656624</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="D5" t="n">
+        <v>83258.8</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.5843260734633019</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.6171764153144865</v>
+      </c>
+      <c r="H5" t="n">
+        <v>-0.001422060304</v>
+      </c>
+      <c r="I5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-09-30 12:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1001.777570656624</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="D6" t="n">
+        <v>83883</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.5861390963416431</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.6175356829013292</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-09-30 16:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1003.291978868766</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="D7" t="n">
+        <v>84104.89999999999</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.5868025583776828</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.6196572376769091</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.038891787858</v>
+      </c>
+      <c r="I7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-09-30 20:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>999.537878868766</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="D8" t="n">
+        <v>83568.60000000001</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.5852506566955277</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.6199931783186496</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-10-01 00:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>999.537475038766</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="D9" t="n">
+        <v>83576.89999999999</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.5853090200318001</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.622285465172533</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.05850383</v>
+      </c>
+      <c r="I9" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -543,21 +996,89 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>info</t>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>bar</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>side</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>qty</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>price</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>fee</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>reason</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>expo_before</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>expo_after</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>sin datos todavía</t>
-        </is>
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-09-29 20:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="E2" t="n">
+        <v>83579.11248</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.29252689368</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>BANDA</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.5851764380923165</v>
       </c>
     </row>
   </sheetData>
@@ -571,21 +1092,119 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:M2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>info</t>
+          <t>posicion</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>abre</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>cierra</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>estado</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>pnl_usdt</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>pnl_pct</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>resultado</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>n_lotes</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>px_entrada_medio</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>mfe_pct</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>mae_pct</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>senal_al_abrir</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>duracion_dias</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>sin datos todavía</t>
-        </is>
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-09-29 20:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>ABIERTA</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>-0.4625249612340667</v>
+      </c>
+      <c r="F2" t="n">
+        <v>-0.000462524961234</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>PIERDE (no realizado)</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I2" t="n">
+        <v>83579.11248</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0.006290896186841</v>
+      </c>
+      <c r="K2" t="n">
+        <v>-0.0038324465347324</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="M2" t="n">
+        <v>1.166666666666667</v>
       </c>
     </row>
   </sheetData>
@@ -599,20 +1218,128 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>info</t>
+          <t>lote</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>abre</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>cierra</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>estado</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>qty</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>px_entrada</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>pnl_usdt</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>pnl_pct</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>resultado</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>funding_pagado</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>mfe_pct</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>mae_pct</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>senal_al_entrar</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>motivo</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>sin datos todavía</t>
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-09-29 20:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>ABIERTO</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="F2" t="n">
+        <v>83579.11248</v>
+      </c>
+      <c r="G2" t="n">
+        <v>-0.4625249612340137</v>
+      </c>
+      <c r="H2" t="n">
+        <v>-0.000790568271203</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>PIERDE (no realizado)</t>
+        </is>
+      </c>
+      <c r="J2" t="n">
+        <v>0.154510707554</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0.006290896186841</v>
+      </c>
+      <c r="L2" t="n">
+        <v>-0.0038324465347324</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>BANDA</t>
         </is>
       </c>
     </row>
@@ -674,20 +1401,20 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0</v>
+        <v>-0.0007663354382617671</v>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>0.006377236760283789</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -706,7 +1433,7 @@
         <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="n">
@@ -729,7 +1456,7 @@
         <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="n">
@@ -752,7 +1479,7 @@
         <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="n">
@@ -775,7 +1502,7 @@
         <v>0</v>
       </c>
       <c r="E6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="n">
@@ -789,16 +1516,16 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0</v>
+        <v>-0.0007555304832757015</v>
       </c>
       <c r="C7" t="n">
-        <v>0</v>
+        <v>0.01005705945566326</v>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="n">
@@ -821,7 +1548,7 @@
         <v>0</v>
       </c>
       <c r="E8" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="n">
@@ -835,16 +1562,16 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0</v>
+        <v>-0.008755142750290323</v>
       </c>
       <c r="C9" t="n">
-        <v>0</v>
+        <v>0.008755142750290323</v>
       </c>
       <c r="D9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="n">
@@ -858,16 +1585,16 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0</v>
+        <v>-0.0007555304832757015</v>
       </c>
       <c r="C10" t="n">
-        <v>0</v>
+        <v>0.01005705945566326</v>
       </c>
       <c r="D10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E10" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="n">
@@ -881,20 +1608,20 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0</v>
+        <v>-0.0045099301825412</v>
       </c>
       <c r="C11" t="n">
-        <v>0</v>
+        <v>0.006377236760283789</v>
       </c>
       <c r="D11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E11" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
@@ -904,16 +1631,16 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0</v>
+        <v>-0.0007555304832757015</v>
       </c>
       <c r="C12" t="n">
-        <v>0</v>
+        <v>0.01005705945566326</v>
       </c>
       <c r="D12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E12" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="n">
@@ -927,16 +1654,16 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0</v>
+        <v>-0.007077236284004473</v>
       </c>
       <c r="C13" t="n">
-        <v>0</v>
+        <v>0.007077236284004473</v>
       </c>
       <c r="D13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E13" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="n">
@@ -950,20 +1677,20 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0</v>
+        <v>-0.0045099301825412</v>
       </c>
       <c r="C14" t="n">
-        <v>0</v>
+        <v>0.006377236760283789</v>
       </c>
       <c r="D14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E14" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
@@ -973,16 +1700,16 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0</v>
+        <v>-0.0007663354382617671</v>
       </c>
       <c r="C15" t="n">
-        <v>0</v>
+        <v>0.006377236760283789</v>
       </c>
       <c r="D15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="n">
@@ -1005,7 +1732,7 @@
         <v>0</v>
       </c>
       <c r="E16" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="n">

</xml_diff>

<commit_message>
mesas + paper: actualización 2026-10-02 08:00
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AtSxiX9NxnepDF7aXKR3KZ
</commit_message>
<xml_diff>
--- a/millonary/paper_state/semanal/diario.xlsx
+++ b/millonary/paper_state/semanal/diario.xlsx
@@ -442,7 +442,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-01 10:11:05.733781+00:00</t>
+          <t>2026-10-02 09:10:46.609269+00:00</t>
         </is>
       </c>
     </row>
@@ -473,7 +473,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>999.537475038766</v>
+        <v>1008.129739068766</v>
       </c>
     </row>
     <row r="6">
@@ -483,7 +483,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>-5.303242508802875e-05</v>
+        <v>0.008542751701033247</v>
       </c>
     </row>
     <row r="7">
@@ -493,7 +493,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>-5.303242508802875e-05</v>
+        <v>0.008542751701033247</v>
       </c>
     </row>
     <row r="8">
@@ -503,7 +503,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.003742184637251178</v>
+        <v>0.00516297454689163</v>
       </c>
     </row>
     <row r="9">
@@ -513,7 +513,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.003742184637251178</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -523,7 +523,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11">
@@ -533,7 +533,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
     </row>
     <row r="12">
@@ -543,7 +543,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.5853090200318001</v>
+        <v>0.5890186322134632</v>
       </c>
     </row>
     <row r="13">
@@ -553,7 +553,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
     </row>
     <row r="14">
@@ -640,7 +640,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>{"dias": 2, "estado": "insuficiente"}</t>
+          <t>{"dias": 3, "estado": "insuficiente"}</t>
         </is>
       </c>
     </row>
@@ -664,7 +664,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Mantener el objetivo del núcleo: 0.62× de exposición.</t>
+          <t>Mantener el objetivo del núcleo: 0.63× de exposición.</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>{"certificadas": [], "forward": {"S01 Parabolic SAR + EMA200": {"retorno": -0.0007663354382617671, "caida_max": 0.006377236760283789, "ops": 1, "dias": 2, "sharpe": null, "posicion_actual": 1.0}, "S02 Ichimoku": {"retorno": 0.0, "caida_max": 0.0, "ops": 0, "dias": 2, "sharpe": null, "posicion_actual": 0.0}, "S03 Bollinger + RSI (reversi\u00f3n)": {"retorno": 0.0, "caida_max": 0.0, "ops": 0, "dias": 2, "sharpe": null, "posicion_actual": 0.0}, "S04 Keltner ruptura": {"retorno": 0.0, "caida_max": 0.0, "ops": 0, "dias": 2, "sharpe": null, "posicion_actual": 0.0}, "S05 RSI(2) retroceso (largo)": {"retorno": 0.0, "caida_max": 0.0, "ops": 0, "dias": 2, "sharpe": null, "posicion_actual": 0.0}, "S06 Cruce SMA 7-25": {"retorno": -0.0007555304832757015, "caida_max": 0.010057059455663264, "ops": 1, "dias": 2, "sharpe": null, "posicion_actual": -1.0}, "S07 SMA 7-25 + filtro 200 (largo)": {"retorno": 0.0, "caida_max": 0.0, "ops": 0, "dias": 2, "sharpe": null, "posicion_actual": 0.0}, "S08 Canal 20 por tercios": {"retorno": -0.008755142750290323, "caida_max": 0.008755142750290323, "ops": 1, "dias": 2, "sharpe": null, "posicion_actual": 0.0}, "S09 Donchian 20/10": {"retorno": -0.0007555304832757015, "caida_max": 0.010057059455663264, "ops": 1, "dias": 2, "sharpe": null, "posicion_actual": -1.0}, "S10 MACD + EMA200": {"retorno": -0.0045099301825412, "caida_max": 0.006377236760283789, "ops": 1, "dias": 2, "sharpe": null, "posicion_actual": 1.0}, "S11 Supertrend 10/3": {"retorno": -0.0007555304832757015, "caida_max": 0.010057059455663264, "ops": 1, "dias": 2, "sharpe": null, "posicion_actual": -1.0}, "S12 Expansi\u00f3n de volatilidad": {"retorno": -0.007077236284004473, "caida_max": 0.007077236284004473, "ops": 1, "dias": 2, "sharpe": null, "posicion_actual": 0.0}, "S13 Retroceso a EMA20": {"retorno": -0.0045099301825412, "caida_max": 0.006377236760283789, "ops": 1, "dias": 2, "sharpe": null, "posicion_actual": 1.0}, "S14 Momentum 90 d": {"retorno": -0.0007663354382617671, "caida_max": 0.006377236760283789, "ops": 1, "dias": 2, "sharpe": null, "posicion_actual": 1.0}, "S15 RSI14 + EMA200": {"retorno": 0.0, "caida_max": 0.0, "ops": 0, "dias": 2, "sharpe": null, "posicion_actual": 0.0}}}</t>
+          <t>{"certificadas": [], "forward": {"S01 Parabolic SAR + EMA200": {"retorno": -0.0038991736216299477, "caida_max": 0.009492483416736697, "ops": 1, "dias": 3, "sharpe": null, "posicion_actual": 0.0}, "S02 Ichimoku": {"retorno": 0.0, "caida_max": 0.0, "ops": 0, "dias": 3, "sharpe": null, "posicion_actual": 1.0}, "S03 Bollinger + RSI (reversi\u00f3n)": {"retorno": 0.0, "caida_max": 0.0, "ops": 0, "dias": 3, "sharpe": null, "posicion_actual": 0.0}, "S04 Keltner ruptura": {"retorno": 0.0, "caida_max": 0.0, "ops": 0, "dias": 3, "sharpe": null, "posicion_actual": 0.0}, "S05 RSI(2) retroceso (largo)": {"retorno": 0.0, "caida_max": 0.0, "ops": 0, "dias": 3, "sharpe": null, "posicion_actual": 0.0}, "S06 Cruce SMA 7-25": {"retorno": 0.005386602181837397, "caida_max": 0.010057059455663264, "ops": 2, "dias": 3, "sharpe": null, "posicion_actual": 1.0}, "S07 SMA 7-25 + filtro 200 (largo)": {"retorno": 0.010435130319854657, "caida_max": 0.0, "ops": 1, "dias": 3, "sharpe": null, "posicion_actual": 1.0}, "S08 Canal 20 por tercios": {"retorno": -0.014501381419916859, "caida_max": 0.016041874299728143, "ops": 3, "dias": 3, "sharpe": null, "posicion_actual": 1.0}, "S09 Donchian 20/10": {"retorno": -0.015320017115938334, "caida_max": 0.018264879276909896, "ops": 1, "dias": 3, "sharpe": null, "posicion_actual": -1.0}, "S10 MACD + EMA200": {"retorno": 0.010108091071524328, "caida_max": 0.008798642466463114, "ops": 1, "dias": 3, "sharpe": null, "posicion_actual": 1.0}, "S11 Supertrend 10/3": {"retorno": -0.015320017115938334, "caida_max": 0.018264879276909896, "ops": 1, "dias": 3, "sharpe": null, "posicion_actual": -1.0}, "S12 Expansi\u00f3n de volatilidad": {"retorno": -0.0062188423978757346, "caida_max": 0.007772282218605708, "ops": 2, "dias": 3, "sharpe": null, "posicion_actual": 0.0}, "S13 Retroceso a EMA20": {"retorno": 0.002724468219000631, "caida_max": 0.009492483416736586, "ops": 2, "dias": 3, "sharpe": null, "posicion_actual": 1.0}, "S14 Momentum 90 d": {"retorno": 0.013906657682623225, "caida_max": 0.008798642466463114, "ops": 1, "dias": 3, "sharpe": null, "posicion_actual": 1.0}, "S15 RSI14 + EMA200": {"retorno": 0.001565608169265209, "caida_max": 0.0, "ops": 1, "dias": 3, "sharpe": null, "posicion_actual": 1.0}}}</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>{"n_pruebas": 75, "etapas": {"descartada (E1/E2)": 54, "E3 sombra": 21}, "adoptables": [], "top_forward": [], "ultima_actualizacion": "2026-10-01 10:11:05.733781+00:00"}</t>
+          <t>{"n_pruebas": 75, "etapas": {"descartada (E1/E2)": 54, "E3 sombra": 21}, "adoptables": [], "top_forward": [], "ultima_actualizacion": "2026-10-02 09:10:46.609269+00:00"}</t>
         </is>
       </c>
     </row>
@@ -703,7 +703,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -984,6 +984,180 @@
         <v>0.05850383</v>
       </c>
       <c r="I9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-10-01 04:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1000.570675038766</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="D10" t="n">
+        <v>83724.5</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.585737234381063</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.6245335491603373</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-10-01 08:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>998.112007918766</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="D11" t="n">
+        <v>83381.60000000001</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.5847752510432713</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.6259555142873255</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0.05836712</v>
+      </c>
+      <c r="I11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-10-01 12:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>1001.588207918766</v>
+      </c>
+      <c r="C12" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="D12" t="n">
+        <v>83878.2</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0.5862163665245754</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0.6270487405972291</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-10-01 16:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>1003.263219788766</v>
+      </c>
+      <c r="C13" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="D13" t="n">
+        <v>84125.89999999999</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.5869659012556916</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0.6291355576294307</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0.05888813</v>
+      </c>
+      <c r="I13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-10-01 20:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>1006.787719788766</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="D14" t="n">
+        <v>84629.39999999999</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0.5884118254087293</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0.6302347745803959</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-10-02 00:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>1008.129739068766</v>
+      </c>
+      <c r="C15" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="D15" t="n">
+        <v>84829.60000000001</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0.5890186322134632</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0.6324433845610925</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0.05938072</v>
+      </c>
+      <c r="I15" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1178,14 +1352,14 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>-0.4625249612340667</v>
+        <v>8.129739068765957</v>
       </c>
       <c r="F2" t="n">
-        <v>-0.000462524961234</v>
+        <v>0.0081297390687659</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>PIERDE (no realizado)</t>
+          <t>GANA (no realizado)</t>
         </is>
       </c>
       <c r="H2" t="n">
@@ -1195,7 +1369,7 @@
         <v>83579.11248</v>
       </c>
       <c r="J2" t="n">
-        <v>0.006290896186841</v>
+        <v>0.0149617228861964</v>
       </c>
       <c r="K2" t="n">
         <v>-0.0038324465347324</v>
@@ -1204,7 +1378,7 @@
         <v>0.875</v>
       </c>
       <c r="M2" t="n">
-        <v>1.166666666666667</v>
+        <v>2.166666666666667</v>
       </c>
     </row>
   </sheetData>
@@ -1315,21 +1489,21 @@
         <v>83579.11248</v>
       </c>
       <c r="G2" t="n">
-        <v>-0.4625249612340137</v>
+        <v>8.129739068766067</v>
       </c>
       <c r="H2" t="n">
-        <v>-0.000790568271203</v>
+        <v>0.0138957122309228</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>PIERDE (no realizado)</t>
+          <t>GANA (no realizado)</t>
         </is>
       </c>
       <c r="J2" t="n">
-        <v>0.154510707554</v>
+        <v>0.331146677554</v>
       </c>
       <c r="K2" t="n">
-        <v>0.006290896186841</v>
+        <v>0.0149617228861964</v>
       </c>
       <c r="L2" t="n">
         <v>-0.0038324465347324</v>
@@ -1401,20 +1575,20 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>-0.0007663354382617671</v>
+        <v>-0.003899173621629948</v>
       </c>
       <c r="C2" t="n">
-        <v>0.006377236760283789</v>
+        <v>0.009492483416736697</v>
       </c>
       <c r="D2" t="n">
         <v>1</v>
       </c>
       <c r="E2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -1433,11 +1607,11 @@
         <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -1456,7 +1630,7 @@
         <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="n">
@@ -1479,7 +1653,7 @@
         <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="n">
@@ -1502,7 +1676,7 @@
         <v>0</v>
       </c>
       <c r="E6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="n">
@@ -1516,20 +1690,20 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>-0.0007555304832757015</v>
+        <v>0.005386602181837397</v>
       </c>
       <c r="C7" t="n">
         <v>0.01005705945566326</v>
       </c>
       <c r="D7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
@@ -1539,20 +1713,20 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0</v>
+        <v>0.01043513031985466</v>
       </c>
       <c r="C8" t="n">
         <v>0</v>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -1562,20 +1736,20 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>-0.008755142750290323</v>
+        <v>-0.01450138141991686</v>
       </c>
       <c r="C9" t="n">
-        <v>0.008755142750290323</v>
+        <v>0.01604187429972814</v>
       </c>
       <c r="D9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -1585,16 +1759,16 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>-0.0007555304832757015</v>
+        <v>-0.01532001711593833</v>
       </c>
       <c r="C10" t="n">
-        <v>0.01005705945566326</v>
+        <v>0.0182648792769099</v>
       </c>
       <c r="D10" t="n">
         <v>1</v>
       </c>
       <c r="E10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="n">
@@ -1608,16 +1782,16 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>-0.0045099301825412</v>
+        <v>0.01010809107152433</v>
       </c>
       <c r="C11" t="n">
-        <v>0.006377236760283789</v>
+        <v>0.008798642466463114</v>
       </c>
       <c r="D11" t="n">
         <v>1</v>
       </c>
       <c r="E11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="n">
@@ -1631,16 +1805,16 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>-0.0007555304832757015</v>
+        <v>-0.01532001711593833</v>
       </c>
       <c r="C12" t="n">
-        <v>0.01005705945566326</v>
+        <v>0.0182648792769099</v>
       </c>
       <c r="D12" t="n">
         <v>1</v>
       </c>
       <c r="E12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="n">
@@ -1654,16 +1828,16 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>-0.007077236284004473</v>
+        <v>-0.006218842397875735</v>
       </c>
       <c r="C13" t="n">
-        <v>0.007077236284004473</v>
+        <v>0.007772282218605708</v>
       </c>
       <c r="D13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E13" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="n">
@@ -1677,16 +1851,16 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>-0.0045099301825412</v>
+        <v>0.002724468219000631</v>
       </c>
       <c r="C14" t="n">
-        <v>0.006377236760283789</v>
+        <v>0.009492483416736586</v>
       </c>
       <c r="D14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E14" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="n">
@@ -1700,16 +1874,16 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>-0.0007663354382617671</v>
+        <v>0.01390665768262322</v>
       </c>
       <c r="C15" t="n">
-        <v>0.006377236760283789</v>
+        <v>0.008798642466463114</v>
       </c>
       <c r="D15" t="n">
         <v>1</v>
       </c>
       <c r="E15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="n">
@@ -1723,20 +1897,20 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0</v>
+        <v>0.001565608169265209</v>
       </c>
       <c r="C16" t="n">
         <v>0</v>
       </c>
       <c r="D16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
paper: resumen semanal regenerado por la rutina diaria
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AtSxiX9NxnepDF7aXKR3KZ
</commit_message>
<xml_diff>
--- a/millonary/paper_state/semanal/diario.xlsx
+++ b/millonary/paper_state/semanal/diario.xlsx
@@ -442,7 +442,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-02 09:10:46.609269+00:00</t>
+          <t>2026-10-02 09:34:24.962435+00:00</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>{"n_pruebas": 75, "etapas": {"descartada (E1/E2)": 54, "E3 sombra": 21}, "adoptables": [], "top_forward": [], "ultima_actualizacion": "2026-10-02 09:10:46.609269+00:00"}</t>
+          <t>{"n_pruebas": 75, "etapas": {"descartada (E1/E2)": 54, "E3 sombra": 21}, "adoptables": [], "top_forward": [], "ultima_actualizacion": "2026-10-02 09:34:24.962435+00:00"}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
paper: actualización diaria 2026-10-03
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AtSxiX9NxnepDF7aXKR3KZ
</commit_message>
<xml_diff>
--- a/millonary/paper_state/semanal/diario.xlsx
+++ b/millonary/paper_state/semanal/diario.xlsx
@@ -442,7 +442,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-02 09:34:24.962435+00:00</t>
+          <t>2026-10-03 04:17:36.656115+00:00</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>{"certificadas": [], "forward": {"S01 Parabolic SAR + EMA200": {"retorno": -0.0038991736216299477, "caida_max": 0.009492483416736697, "ops": 1, "dias": 3, "sharpe": null, "posicion_actual": 0.0}, "S02 Ichimoku": {"retorno": 0.0, "caida_max": 0.0, "ops": 0, "dias": 3, "sharpe": null, "posicion_actual": 1.0}, "S03 Bollinger + RSI (reversi\u00f3n)": {"retorno": 0.0, "caida_max": 0.0, "ops": 0, "dias": 3, "sharpe": null, "posicion_actual": 0.0}, "S04 Keltner ruptura": {"retorno": 0.0, "caida_max": 0.0, "ops": 0, "dias": 3, "sharpe": null, "posicion_actual": 0.0}, "S05 RSI(2) retroceso (largo)": {"retorno": 0.0, "caida_max": 0.0, "ops": 0, "dias": 3, "sharpe": null, "posicion_actual": 0.0}, "S06 Cruce SMA 7-25": {"retorno": 0.005386602181837397, "caida_max": 0.010057059455663264, "ops": 2, "dias": 3, "sharpe": null, "posicion_actual": 1.0}, "S07 SMA 7-25 + filtro 200 (largo)": {"retorno": 0.010435130319854657, "caida_max": 0.0, "ops": 1, "dias": 3, "sharpe": null, "posicion_actual": 1.0}, "S08 Canal 20 por tercios": {"retorno": -0.014501381419916859, "caida_max": 0.016041874299728143, "ops": 3, "dias": 3, "sharpe": null, "posicion_actual": 1.0}, "S09 Donchian 20/10": {"retorno": -0.015320017115938334, "caida_max": 0.018264879276909896, "ops": 1, "dias": 3, "sharpe": null, "posicion_actual": -1.0}, "S10 MACD + EMA200": {"retorno": 0.010108091071524328, "caida_max": 0.008798642466463114, "ops": 1, "dias": 3, "sharpe": null, "posicion_actual": 1.0}, "S11 Supertrend 10/3": {"retorno": -0.015320017115938334, "caida_max": 0.018264879276909896, "ops": 1, "dias": 3, "sharpe": null, "posicion_actual": -1.0}, "S12 Expansi\u00f3n de volatilidad": {"retorno": -0.0062188423978757346, "caida_max": 0.007772282218605708, "ops": 2, "dias": 3, "sharpe": null, "posicion_actual": 0.0}, "S13 Retroceso a EMA20": {"retorno": 0.002724468219000631, "caida_max": 0.009492483416736586, "ops": 2, "dias": 3, "sharpe": null, "posicion_actual": 1.0}, "S14 Momentum 90 d": {"retorno": 0.013906657682623225, "caida_max": 0.008798642466463114, "ops": 1, "dias": 3, "sharpe": null, "posicion_actual": 1.0}, "S15 RSI14 + EMA200": {"retorno": 0.001565608169265209, "caida_max": 0.0, "ops": 1, "dias": 3, "sharpe": null, "posicion_actual": 1.0}}}</t>
+          <t>{"certificadas": [], "forward": {"S01 Parabolic SAR + EMA200": {"retorno": -0.003818821648301718, "caida_max": 0.009412582636166844, "ops": 1, "dias": 3, "sharpe": null, "posicion_actual": 0.0}, "S02 Ichimoku": {"retorno": 0.0, "caida_max": 0.0, "ops": 0, "dias": 3, "sharpe": null, "posicion_actual": 1.0}, "S03 Bollinger + RSI (reversi\u00f3n)": {"retorno": 0.0, "caida_max": 0.0, "ops": 0, "dias": 3, "sharpe": null, "posicion_actual": 0.0}, "S04 Keltner ruptura": {"retorno": 0.0, "caida_max": 0.0, "ops": 0, "dias": 3, "sharpe": null, "posicion_actual": 0.0}, "S05 RSI(2) retroceso (largo)": {"retorno": 0.0, "caida_max": 0.0, "ops": 0, "dias": 3, "sharpe": null, "posicion_actual": 0.0}, "S06 Cruce SMA 7-25": {"retorno": 0.00541285478297282, "caida_max": 0.010057059455663264, "ops": 2, "dias": 3, "sharpe": null, "posicion_actual": 1.0}, "S07 SMA 7-25 + filtro 200 (largo)": {"retorno": 0.010542510629850232, "caida_max": 0.0, "ops": 1, "dias": 3, "sharpe": null, "posicion_actual": 1.0}, "S08 Canal 20 por tercios": {"retorno": -0.01443023395662224, "caida_max": 0.016041874299728143, "ops": 3, "dias": 3, "sharpe": null, "posicion_actual": 1.0}, "S09 Donchian 20/10": {"retorno": -0.015504084875667234, "caida_max": 0.018448396548977675, "ops": 1, "dias": 3, "sharpe": null, "posicion_actual": -1.0}, "S10 MACD + EMA200": {"retorno": 0.010296903112296363, "caida_max": 0.008718685716168184, "ops": 1, "dias": 3, "sharpe": null, "posicion_actual": 1.0}, "S11 Supertrend 10/3": {"retorno": -0.015504084875667234, "caida_max": 0.018448396548977675, "ops": 1, "dias": 3, "sharpe": null, "posicion_actual": -1.0}, "S12 Expansi\u00f3n de volatilidad": {"retorno": -0.006125106611438724, "caida_max": 0.007750327807717339, "ops": 2, "dias": 3, "sharpe": null, "posicion_actual": 0.0}, "S13 Retroceso a EMA20": {"retorno": 0.002911923981757214, "caida_max": 0.009412582636166844, "ops": 2, "dias": 3, "sharpe": null, "posicion_actual": 1.0}, "S14 Momentum 90 d": {"retorno": 0.014096179761380778, "caida_max": 0.008718685716168073, "ops": 1, "dias": 3, "sharpe": null, "posicion_actual": 1.0}, "S15 RSI14 + EMA200": {"retorno": 0.0016379155789367772, "caida_max": 0.0, "ops": 1, "dias": 3, "sharpe": null, "posicion_actual": 1.0}}}</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>{"n_pruebas": 75, "etapas": {"descartada (E1/E2)": 54, "E3 sombra": 21}, "adoptables": [], "top_forward": [], "ultima_actualizacion": "2026-10-02 09:34:24.962435+00:00"}</t>
+          <t>{"n_pruebas": 75, "etapas": {"descartada (E1/E2)": 54, "E3 sombra": 21}, "adoptables": [], "top_forward": [], "ultima_actualizacion": "2026-10-03 04:17:36.656115+00:00"}</t>
         </is>
       </c>
     </row>
@@ -1575,10 +1575,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>-0.003899173621629948</v>
+        <v>-0.003818821648301718</v>
       </c>
       <c r="C2" t="n">
-        <v>0.009492483416736697</v>
+        <v>0.009412582636166844</v>
       </c>
       <c r="D2" t="n">
         <v>1</v>
@@ -1690,7 +1690,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.005386602181837397</v>
+        <v>0.00541285478297282</v>
       </c>
       <c r="C7" t="n">
         <v>0.01005705945566326</v>
@@ -1713,7 +1713,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.01043513031985466</v>
+        <v>0.01054251062985023</v>
       </c>
       <c r="C8" t="n">
         <v>0</v>
@@ -1736,7 +1736,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>-0.01450138141991686</v>
+        <v>-0.01443023395662224</v>
       </c>
       <c r="C9" t="n">
         <v>0.01604187429972814</v>
@@ -1759,10 +1759,10 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>-0.01532001711593833</v>
+        <v>-0.01550408487566723</v>
       </c>
       <c r="C10" t="n">
-        <v>0.0182648792769099</v>
+        <v>0.01844839654897767</v>
       </c>
       <c r="D10" t="n">
         <v>1</v>
@@ -1782,10 +1782,10 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.01010809107152433</v>
+        <v>0.01029690311229636</v>
       </c>
       <c r="C11" t="n">
-        <v>0.008798642466463114</v>
+        <v>0.008718685716168184</v>
       </c>
       <c r="D11" t="n">
         <v>1</v>
@@ -1805,10 +1805,10 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>-0.01532001711593833</v>
+        <v>-0.01550408487566723</v>
       </c>
       <c r="C12" t="n">
-        <v>0.0182648792769099</v>
+        <v>0.01844839654897767</v>
       </c>
       <c r="D12" t="n">
         <v>1</v>
@@ -1828,10 +1828,10 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>-0.006218842397875735</v>
+        <v>-0.006125106611438724</v>
       </c>
       <c r="C13" t="n">
-        <v>0.007772282218605708</v>
+        <v>0.007750327807717339</v>
       </c>
       <c r="D13" t="n">
         <v>2</v>
@@ -1851,10 +1851,10 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.002724468219000631</v>
+        <v>0.002911923981757214</v>
       </c>
       <c r="C14" t="n">
-        <v>0.009492483416736586</v>
+        <v>0.009412582636166844</v>
       </c>
       <c r="D14" t="n">
         <v>2</v>
@@ -1874,10 +1874,10 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.01390665768262322</v>
+        <v>0.01409617976138078</v>
       </c>
       <c r="C15" t="n">
-        <v>0.008798642466463114</v>
+        <v>0.008718685716168073</v>
       </c>
       <c r="D15" t="n">
         <v>1</v>
@@ -1897,7 +1897,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.001565608169265209</v>
+        <v>0.001637915578936777</v>
       </c>
       <c r="C16" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
paper: actualización diaria 2026-10-04
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AtSxiX9NxnepDF7aXKR3KZ
</commit_message>
<xml_diff>
--- a/millonary/paper_state/semanal/diario.xlsx
+++ b/millonary/paper_state/semanal/diario.xlsx
@@ -442,7 +442,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-03 04:17:36.656115+00:00</t>
+          <t>2026-10-04 04:17:40.017359+00:00</t>
         </is>
       </c>
     </row>
@@ -473,7 +473,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1008.129739068766</v>
+        <v>1005.730437336485</v>
       </c>
     </row>
     <row r="6">
@@ -483,7 +483,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.008542751701033247</v>
+        <v>0.006142467017961284</v>
       </c>
     </row>
     <row r="7">
@@ -493,7 +493,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.008542751701033247</v>
+        <v>0.006142467017961284</v>
       </c>
     </row>
     <row r="8">
@@ -503,7 +503,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.00516297454689163</v>
+        <v>0.01450074688943914</v>
       </c>
     </row>
     <row r="9">
@@ -513,7 +513,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0</v>
+        <v>0.01304550293290685</v>
       </c>
     </row>
     <row r="10">
@@ -523,7 +523,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11">
@@ -533,7 +533,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>14</v>
+        <v>20</v>
       </c>
     </row>
     <row r="12">
@@ -543,7 +543,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.5890186322134632</v>
+        <v>0.5880100452822863</v>
       </c>
     </row>
     <row r="13">
@@ -553,7 +553,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>14</v>
+        <v>20</v>
       </c>
     </row>
     <row r="14">
@@ -628,7 +628,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>{"G1_replica": false, "G2_integridad": true, "G3_envolvente": true, "G4_no_anomalo": true, "G5_registro_cuadra": true}</t>
+          <t>{"G1_replica": true, "G2_integridad": true, "G3_envolvente": true, "G4_no_anomalo": true, "G5_registro_cuadra": true}</t>
         </is>
       </c>
     </row>
@@ -640,7 +640,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>{"dias": 3, "estado": "insuficiente"}</t>
+          <t>{"dias": 4, "estado": "insuficiente"}</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>{"certificadas": [], "forward": {"S01 Parabolic SAR + EMA200": {"retorno": -0.003818821648301718, "caida_max": 0.009412582636166844, "ops": 1, "dias": 3, "sharpe": null, "posicion_actual": 0.0}, "S02 Ichimoku": {"retorno": 0.0, "caida_max": 0.0, "ops": 0, "dias": 3, "sharpe": null, "posicion_actual": 1.0}, "S03 Bollinger + RSI (reversi\u00f3n)": {"retorno": 0.0, "caida_max": 0.0, "ops": 0, "dias": 3, "sharpe": null, "posicion_actual": 0.0}, "S04 Keltner ruptura": {"retorno": 0.0, "caida_max": 0.0, "ops": 0, "dias": 3, "sharpe": null, "posicion_actual": 0.0}, "S05 RSI(2) retroceso (largo)": {"retorno": 0.0, "caida_max": 0.0, "ops": 0, "dias": 3, "sharpe": null, "posicion_actual": 0.0}, "S06 Cruce SMA 7-25": {"retorno": 0.00541285478297282, "caida_max": 0.010057059455663264, "ops": 2, "dias": 3, "sharpe": null, "posicion_actual": 1.0}, "S07 SMA 7-25 + filtro 200 (largo)": {"retorno": 0.010542510629850232, "caida_max": 0.0, "ops": 1, "dias": 3, "sharpe": null, "posicion_actual": 1.0}, "S08 Canal 20 por tercios": {"retorno": -0.01443023395662224, "caida_max": 0.016041874299728143, "ops": 3, "dias": 3, "sharpe": null, "posicion_actual": 1.0}, "S09 Donchian 20/10": {"retorno": -0.015504084875667234, "caida_max": 0.018448396548977675, "ops": 1, "dias": 3, "sharpe": null, "posicion_actual": -1.0}, "S10 MACD + EMA200": {"retorno": 0.010296903112296363, "caida_max": 0.008718685716168184, "ops": 1, "dias": 3, "sharpe": null, "posicion_actual": 1.0}, "S11 Supertrend 10/3": {"retorno": -0.015504084875667234, "caida_max": 0.018448396548977675, "ops": 1, "dias": 3, "sharpe": null, "posicion_actual": -1.0}, "S12 Expansi\u00f3n de volatilidad": {"retorno": -0.006125106611438724, "caida_max": 0.007750327807717339, "ops": 2, "dias": 3, "sharpe": null, "posicion_actual": 0.0}, "S13 Retroceso a EMA20": {"retorno": 0.002911923981757214, "caida_max": 0.009412582636166844, "ops": 2, "dias": 3, "sharpe": null, "posicion_actual": 1.0}, "S14 Momentum 90 d": {"retorno": 0.014096179761380778, "caida_max": 0.008718685716168073, "ops": 1, "dias": 3, "sharpe": null, "posicion_actual": 1.0}, "S15 RSI14 + EMA200": {"retorno": 0.0016379155789367772, "caida_max": 0.0, "ops": 1, "dias": 3, "sharpe": null, "posicion_actual": 1.0}}}</t>
+          <t>{"certificadas": [], "forward": {"S01 Parabolic SAR + EMA200": {"retorno": -0.016241403929057596, "caida_max": 0.024438765486139102, "ops": 2, "dias": 4, "sharpe": null, "posicion_actual": 1.0}, "S02 Ichimoku": {"retorno": -0.004937674929030522, "caida_max": 0.024438765486139102, "ops": 1, "dias": 4, "sharpe": null, "posicion_actual": 1.0}, "S03 Bollinger + RSI (reversi\u00f3n)": {"retorno": 0.021458005192262375, "caida_max": 0.0025141225519644816, "ops": 1, "dias": 4, "sharpe": null, "posicion_actual": -1.0}, "S04 Keltner ruptura": {"retorno": -0.02581271738866342, "caida_max": 0.02581271738866342, "ops": 1, "dias": 4, "sharpe": null, "posicion_actual": 0.0}, "S05 RSI(2) retroceso (largo)": {"retorno": 0.0, "caida_max": 0.0, "ops": 0, "dias": 4, "sharpe": null, "posicion_actual": 0.0}, "S06 Cruce SMA 7-25": {"retorno": 0.0011439491135745161, "caida_max": 0.024438765486139102, "ops": 2, "dias": 4, "sharpe": null, "posicion_actual": 1.0}, "S07 SMA 7-25 + filtro 200 (largo)": {"retorno": 0.006251824836175146, "caida_max": 0.02443876548613899, "ops": 1, "dias": 4, "sharpe": null, "posicion_actual": 1.0}, "S08 Canal 20 por tercios": {"retorno": -0.012981015998491774, "caida_max": 0.016371566737423682, "ops": 4, "dias": 4, "sharpe": null, "posicion_actual": 0.0}, "S09 Donchian 20/10": {"retorno": -0.04884871046144057, "caida_max": 0.05407147927571376, "ops": 2, "dias": 4, "sharpe": null, "posicion_actual": 1.0}, "S10 MACD + EMA200": {"retorno": 0.006007260149254456, "caida_max": 0.024438765486139102, "ops": 1, "dias": 4, "sharpe": null, "posicion_actual": 1.0}, "S11 Supertrend 10/3": {"retorno": -0.03586740171412017, "caida_max": 0.0411614508549194, "ops": 2, "dias": 4, "sharpe": null, "posicion_actual": 1.0}, "S12 Expansi\u00f3n de volatilidad": {"retorno": -0.01920596579843037, "caida_max": 0.024438765486139102, "ops": 3, "dias": 4, "sharpe": null, "posicion_actual": 1.0}, "S13 Retroceso a EMA20": {"retorno": -0.0013463629277700173, "caida_max": 0.02443876548613899, "ops": 2, "dias": 4, "sharpe": null, "posicion_actual": 1.0}, "S14 Momentum 90 d": {"retorno": 0.009790405361835397, "caida_max": 0.02443876548613899, "ops": 1, "dias": 4, "sharpe": null, "posicion_actual": 1.0}, "S15 RSI14 + EMA200": {"retorno": -0.0026149619888782283, "caida_max": 0.024438765486139213, "ops": 1, "dias": 4, "sharpe": null, "posicion_actual": 1.0}}}</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>{"n_pruebas": 75, "etapas": {"descartada (E1/E2)": 54, "E3 sombra": 21}, "adoptables": [], "top_forward": [], "ultima_actualizacion": "2026-10-03 04:17:36.656115+00:00"}</t>
+          <t>{"n_pruebas": 75, "etapas": {"descartada (E1/E2)": 54, "E3 sombra": 21}, "adoptables": [], "top_forward": [], "ultima_actualizacion": "2026-10-04 04:17:40.017359+00:00"}</t>
         </is>
       </c>
     </row>
@@ -703,7 +703,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1158,6 +1158,180 @@
         <v>0.05938072</v>
       </c>
       <c r="I15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-10-02 04:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>1012.782264485809</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="D16" t="n">
+        <v>85476.60000000001</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0.5907846345470673</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0.6326932837811364</v>
+      </c>
+      <c r="H16" t="n">
+        <v>-0.1235254170432</v>
+      </c>
+      <c r="I16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-10-02 08:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>1016.835919475809</v>
+      </c>
+      <c r="C17" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="D17" t="n">
+        <v>86064.3</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0.5924752346578888</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0.6333942553345733</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0.06024501</v>
+      </c>
+      <c r="I17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-10-02 12:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>1019.024119475809</v>
+      </c>
+      <c r="C18" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="D18" t="n">
+        <v>86376.89999999999</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0.5933503323856837</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0.6353803202854788</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-10-02 16:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>1011.461008645057</v>
+      </c>
+      <c r="C19" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="D19" t="n">
+        <v>85297.39999999999</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0.5903161811445848</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0.6302081433574255</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0.0066108307520817</v>
+      </c>
+      <c r="I19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-10-02 20:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>1004.247508645057</v>
+      </c>
+      <c r="C20" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="D20" t="n">
+        <v>84266.89999999999</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0.5873734262939397</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0.6257473694606688</v>
+      </c>
+      <c r="H20" t="n">
+        <v>0</v>
+      </c>
+      <c r="I20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-10-03 00:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>1005.730437336485</v>
+      </c>
+      <c r="C21" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="D21" t="n">
+        <v>84482.8</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0.5880100452822863</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0.6279019770277655</v>
+      </c>
+      <c r="H21" t="n">
+        <v>0.0283713085722113</v>
+      </c>
+      <c r="I21" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1352,10 +1526,10 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>8.129739068765957</v>
+        <v>5.730437336484783</v>
       </c>
       <c r="F2" t="n">
-        <v>0.0081297390687659</v>
+        <v>0.0057304373364847</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -1369,7 +1543,7 @@
         <v>83579.11248</v>
       </c>
       <c r="J2" t="n">
-        <v>0.0149617228861964</v>
+        <v>0.033474721577948</v>
       </c>
       <c r="K2" t="n">
         <v>-0.0038324465347324</v>
@@ -1378,7 +1552,7 @@
         <v>0.875</v>
       </c>
       <c r="M2" t="n">
-        <v>2.166666666666667</v>
+        <v>3.166666666666667</v>
       </c>
     </row>
   </sheetData>
@@ -1489,10 +1663,10 @@
         <v>83579.11248</v>
       </c>
       <c r="G2" t="n">
-        <v>8.129739068766067</v>
+        <v>5.730437336484955</v>
       </c>
       <c r="H2" t="n">
-        <v>0.0138957122309228</v>
+        <v>0.009794718810971201</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -1500,10 +1674,10 @@
         </is>
       </c>
       <c r="J2" t="n">
-        <v>0.331146677554</v>
+        <v>0.3028484098350931</v>
       </c>
       <c r="K2" t="n">
-        <v>0.0149617228861964</v>
+        <v>0.033474721577948</v>
       </c>
       <c r="L2" t="n">
         <v>-0.0038324465347324</v>
@@ -1575,20 +1749,20 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>-0.003818821648301718</v>
+        <v>-0.0162414039290576</v>
       </c>
       <c r="C2" t="n">
-        <v>0.009412582636166844</v>
+        <v>0.0244387654861391</v>
       </c>
       <c r="D2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -1598,16 +1772,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0</v>
+        <v>-0.004937674929030522</v>
       </c>
       <c r="C3" t="n">
-        <v>0</v>
+        <v>0.0244387654861391</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="n">
@@ -1621,20 +1795,20 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0</v>
+        <v>0.02145800519226237</v>
       </c>
       <c r="C4" t="n">
-        <v>0</v>
+        <v>0.002514122551964482</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="5">
@@ -1644,16 +1818,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0</v>
+        <v>-0.02581271738866342</v>
       </c>
       <c r="C5" t="n">
-        <v>0</v>
+        <v>0.02581271738866342</v>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="n">
@@ -1676,7 +1850,7 @@
         <v>0</v>
       </c>
       <c r="E6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="n">
@@ -1690,16 +1864,16 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.00541285478297282</v>
+        <v>0.001143949113574516</v>
       </c>
       <c r="C7" t="n">
-        <v>0.01005705945566326</v>
+        <v>0.0244387654861391</v>
       </c>
       <c r="D7" t="n">
         <v>2</v>
       </c>
       <c r="E7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="n">
@@ -1713,16 +1887,16 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.01054251062985023</v>
+        <v>0.006251824836175146</v>
       </c>
       <c r="C8" t="n">
-        <v>0</v>
+        <v>0.02443876548613899</v>
       </c>
       <c r="D8" t="n">
         <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="n">
@@ -1736,20 +1910,20 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>-0.01443023395662224</v>
+        <v>-0.01298101599849177</v>
       </c>
       <c r="C9" t="n">
-        <v>0.01604187429972814</v>
+        <v>0.01637156673742368</v>
       </c>
       <c r="D9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -1759,20 +1933,20 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>-0.01550408487566723</v>
+        <v>-0.04884871046144057</v>
       </c>
       <c r="C10" t="n">
-        <v>0.01844839654897767</v>
+        <v>0.05407147927571376</v>
       </c>
       <c r="D10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
@@ -1782,16 +1956,16 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.01029690311229636</v>
+        <v>0.006007260149254456</v>
       </c>
       <c r="C11" t="n">
-        <v>0.008718685716168184</v>
+        <v>0.0244387654861391</v>
       </c>
       <c r="D11" t="n">
         <v>1</v>
       </c>
       <c r="E11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="n">
@@ -1805,20 +1979,20 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>-0.01550408487566723</v>
+        <v>-0.03586740171412017</v>
       </c>
       <c r="C12" t="n">
-        <v>0.01844839654897767</v>
+        <v>0.0411614508549194</v>
       </c>
       <c r="D12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E12" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -1828,20 +2002,20 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>-0.006125106611438724</v>
+        <v>-0.01920596579843037</v>
       </c>
       <c r="C13" t="n">
-        <v>0.007750327807717339</v>
+        <v>0.0244387654861391</v>
       </c>
       <c r="D13" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E13" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -1851,16 +2025,16 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.002911923981757214</v>
+        <v>-0.001346362927770017</v>
       </c>
       <c r="C14" t="n">
-        <v>0.009412582636166844</v>
+        <v>0.02443876548613899</v>
       </c>
       <c r="D14" t="n">
         <v>2</v>
       </c>
       <c r="E14" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="n">
@@ -1874,16 +2048,16 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.01409617976138078</v>
+        <v>0.009790405361835397</v>
       </c>
       <c r="C15" t="n">
-        <v>0.008718685716168073</v>
+        <v>0.02443876548613899</v>
       </c>
       <c r="D15" t="n">
         <v>1</v>
       </c>
       <c r="E15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="n">
@@ -1897,16 +2071,16 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.001637915578936777</v>
+        <v>-0.002614961988878228</v>
       </c>
       <c r="C16" t="n">
-        <v>0</v>
+        <v>0.02443876548613921</v>
       </c>
       <c r="D16" t="n">
         <v>1</v>
       </c>
       <c r="E16" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="n">

</xml_diff>

<commit_message>
paper: actualización diaria 2026-10-05
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AtSxiX9NxnepDF7aXKR3KZ
</commit_message>
<xml_diff>
--- a/millonary/paper_state/semanal/diario.xlsx
+++ b/millonary/paper_state/semanal/diario.xlsx
@@ -442,7 +442,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-04 04:17:40.017359+00:00</t>
+          <t>2026-10-05 04:17:47.927392+00:00</t>
         </is>
       </c>
     </row>
@@ -473,7 +473,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1005.730437336485</v>
+        <v>1007.304778603525</v>
       </c>
     </row>
     <row r="6">
@@ -483,7 +483,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.006142467017961284</v>
+        <v>0.007717453264318941</v>
       </c>
     </row>
     <row r="7">
@@ -493,7 +493,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.006142467017961284</v>
+        <v>0.007717453264318941</v>
       </c>
     </row>
     <row r="8">
@@ -513,7 +513,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.01304550293290685</v>
+        <v>0.01150055297838537</v>
       </c>
     </row>
     <row r="10">
@@ -523,7 +523,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11">
@@ -533,7 +533,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>20</v>
+        <v>26</v>
       </c>
     </row>
     <row r="12">
@@ -543,7 +543,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.5880100452822863</v>
+        <v>0.5886740662762154</v>
       </c>
     </row>
     <row r="13">
@@ -553,7 +553,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>20</v>
+        <v>26</v>
       </c>
     </row>
     <row r="14">
@@ -640,7 +640,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>{"dias": 4, "estado": "insuficiente"}</t>
+          <t>{"dias": 5, "estado": "insuficiente"}</t>
         </is>
       </c>
     </row>
@@ -664,7 +664,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Mantener el objetivo del núcleo: 0.63× de exposición.</t>
+          <t>Mantener el objetivo del núcleo: 0.64× de exposición.</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>{"certificadas": [], "forward": {"S01 Parabolic SAR + EMA200": {"retorno": -0.016241403929057596, "caida_max": 0.024438765486139102, "ops": 2, "dias": 4, "sharpe": null, "posicion_actual": 1.0}, "S02 Ichimoku": {"retorno": -0.004937674929030522, "caida_max": 0.024438765486139102, "ops": 1, "dias": 4, "sharpe": null, "posicion_actual": 1.0}, "S03 Bollinger + RSI (reversi\u00f3n)": {"retorno": 0.021458005192262375, "caida_max": 0.0025141225519644816, "ops": 1, "dias": 4, "sharpe": null, "posicion_actual": -1.0}, "S04 Keltner ruptura": {"retorno": -0.02581271738866342, "caida_max": 0.02581271738866342, "ops": 1, "dias": 4, "sharpe": null, "posicion_actual": 0.0}, "S05 RSI(2) retroceso (largo)": {"retorno": 0.0, "caida_max": 0.0, "ops": 0, "dias": 4, "sharpe": null, "posicion_actual": 0.0}, "S06 Cruce SMA 7-25": {"retorno": 0.0011439491135745161, "caida_max": 0.024438765486139102, "ops": 2, "dias": 4, "sharpe": null, "posicion_actual": 1.0}, "S07 SMA 7-25 + filtro 200 (largo)": {"retorno": 0.006251824836175146, "caida_max": 0.02443876548613899, "ops": 1, "dias": 4, "sharpe": null, "posicion_actual": 1.0}, "S08 Canal 20 por tercios": {"retorno": -0.012981015998491774, "caida_max": 0.016371566737423682, "ops": 4, "dias": 4, "sharpe": null, "posicion_actual": 0.0}, "S09 Donchian 20/10": {"retorno": -0.04884871046144057, "caida_max": 0.05407147927571376, "ops": 2, "dias": 4, "sharpe": null, "posicion_actual": 1.0}, "S10 MACD + EMA200": {"retorno": 0.006007260149254456, "caida_max": 0.024438765486139102, "ops": 1, "dias": 4, "sharpe": null, "posicion_actual": 1.0}, "S11 Supertrend 10/3": {"retorno": -0.03586740171412017, "caida_max": 0.0411614508549194, "ops": 2, "dias": 4, "sharpe": null, "posicion_actual": 1.0}, "S12 Expansi\u00f3n de volatilidad": {"retorno": -0.01920596579843037, "caida_max": 0.024438765486139102, "ops": 3, "dias": 4, "sharpe": null, "posicion_actual": 1.0}, "S13 Retroceso a EMA20": {"retorno": -0.0013463629277700173, "caida_max": 0.02443876548613899, "ops": 2, "dias": 4, "sharpe": null, "posicion_actual": 1.0}, "S14 Momentum 90 d": {"retorno": 0.009790405361835397, "caida_max": 0.02443876548613899, "ops": 1, "dias": 4, "sharpe": null, "posicion_actual": 1.0}, "S15 RSI14 + EMA200": {"retorno": -0.0026149619888782283, "caida_max": 0.024438765486139213, "ops": 1, "dias": 4, "sharpe": null, "posicion_actual": 1.0}}}</t>
+          <t>{"certificadas": [], "forward": {"S01 Parabolic SAR + EMA200": {"retorno": -0.013622321597007492, "caida_max": 0.024438765486139102, "ops": 2, "dias": 5, "sharpe": null, "posicion_actual": 0.0}, "S02 Ichimoku": {"retorno": -0.0022884984285242993, "caida_max": 0.024438765486139102, "ops": 1, "dias": 5, "sharpe": null, "posicion_actual": 1.0}, "S03 Bollinger + RSI (reversi\u00f3n)": {"retorno": 0.018729435448709753, "caida_max": 0.006622656008078431, "ops": 1, "dias": 5, "sharpe": null, "posicion_actual": -1.0}, "S04 Keltner ruptura": {"retorno": -0.02581271738866342, "caida_max": 0.02581271738866342, "ops": 1, "dias": 5, "sharpe": null, "posicion_actual": 0.0}, "S05 RSI(2) retroceso (largo)": {"retorno": 0.0, "caida_max": 0.0, "ops": 0, "dias": 5, "sharpe": null, "posicion_actual": 0.0}, "S06 Cruce SMA 7-25": {"retorno": 0.0038093168566717406, "caida_max": 0.024438765486139102, "ops": 2, "dias": 5, "sharpe": null, "posicion_actual": 1.0}, "S07 SMA 7-25 + filtro 200 (largo)": {"retorno": 0.008930791390111326, "caida_max": 0.02443876548613899, "ops": 1, "dias": 5, "sharpe": null, "posicion_actual": 1.0}, "S08 Canal 20 por tercios": {"retorno": -0.013671929287292883, "caida_max": 0.01706010664070745, "ops": 4, "dias": 5, "sharpe": null, "posicion_actual": 0.0}, "S09 Donchian 20/10": {"retorno": -0.04631643928486684, "caida_max": 0.05407147927571376, "ops": 2, "dias": 5, "sharpe": null, "posicion_actual": 1.0}, "S10 MACD + EMA200": {"retorno": 0.005613788697409028, "caida_max": 0.024438765486139102, "ops": 1, "dias": 5, "sharpe": null, "posicion_actual": 0.0}, "S11 Supertrend 10/3": {"retorno": -0.03330057011131715, "caida_max": 0.0411614508549194, "ops": 2, "dias": 5, "sharpe": null, "posicion_actual": 1.0}, "S12 Expansi\u00f3n de volatilidad": {"retorno": -0.01814174437269811, "caida_max": 0.024438765486139102, "ops": 3, "dias": 5, "sharpe": null, "posicion_actual": 0.0}, "S13 Retroceso a EMA20": {"retorno": 0.0013123748023395887, "caida_max": 0.02443876548613899, "ops": 2, "dias": 5, "sharpe": null, "posicion_actual": 1.0}, "S14 Momentum 90 d": {"retorno": 0.012478792757198098, "caida_max": 0.02443876548613899, "ops": 1, "dias": 5, "sharpe": null, "posicion_actual": 1.0}, "S15 RSI14 + EMA200": {"retorno": 4.03983218109083e-05, "caida_max": 0.024438765486139213, "ops": 1, "dias": 5, "sharpe": null, "posicion_actual": 1.0}}}</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>{"n_pruebas": 75, "etapas": {"descartada (E1/E2)": 54, "E3 sombra": 21}, "adoptables": [], "top_forward": [], "ultima_actualizacion": "2026-10-04 04:17:40.017359+00:00"}</t>
+          <t>{"n_pruebas": 75, "etapas": {"descartada (E1/E2)": 54, "E3 sombra": 21}, "adoptables": [], "top_forward": [], "ultima_actualizacion": "2026-10-05 04:17:47.927392+00:00"}</t>
         </is>
       </c>
     </row>
@@ -703,7 +703,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:I27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1332,6 +1332,180 @@
         <v>0.0283713085722113</v>
       </c>
       <c r="I21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-10-03 04:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>1006.944937336485</v>
+      </c>
+      <c r="C22" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="D22" t="n">
+        <v>84656.3</v>
+      </c>
+      <c r="E22" t="n">
+        <v>0.5885069560680222</v>
+      </c>
+      <c r="F22" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="G22" t="n">
+        <v>0.6301395972177818</v>
+      </c>
+      <c r="H22" t="n">
+        <v>0</v>
+      </c>
+      <c r="I22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-10-03 08:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>1005.913234211455</v>
+      </c>
+      <c r="C23" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="D23" t="n">
+        <v>84509.3</v>
+      </c>
+      <c r="E23" t="n">
+        <v>0.588087600282676</v>
+      </c>
+      <c r="F23" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0.6322483647156796</v>
+      </c>
+      <c r="H23" t="n">
+        <v>0.0027031250298021</v>
+      </c>
+      <c r="I23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-10-03 12:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>1006.786834211455</v>
+      </c>
+      <c r="C24" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="D24" t="n">
+        <v>84634.10000000001</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0.5884450211985692</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="G24" t="n">
+        <v>0.6345588250675961</v>
+      </c>
+      <c r="H24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-10-03 16:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>1008.167464725298</v>
+      </c>
+      <c r="C25" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="D25" t="n">
+        <v>84835.2</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0.5890354735478486</v>
+      </c>
+      <c r="F25" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="G25" t="n">
+        <v>0.636772250032881</v>
+      </c>
+      <c r="H25" t="n">
+        <v>0.027069486156805</v>
+      </c>
+      <c r="I25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-10-03 20:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>1007.883264725298</v>
+      </c>
+      <c r="C26" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="D26" t="n">
+        <v>84794.60000000001</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0.5889195909625281</v>
+      </c>
+      <c r="F26" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="G26" t="n">
+        <v>0.6390850724813826</v>
+      </c>
+      <c r="H26" t="n">
+        <v>0</v>
+      </c>
+      <c r="I26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-10-04 00:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>1007.304778603525</v>
+      </c>
+      <c r="C27" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="D27" t="n">
+        <v>84710.60000000001</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0.5886740662762154</v>
+      </c>
+      <c r="F27" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="G27" t="n">
+        <v>0.6413468722934025</v>
+      </c>
+      <c r="H27" t="n">
+        <v>-0.0095138782269807</v>
+      </c>
+      <c r="I27" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1526,10 +1700,10 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>5.730437336484783</v>
+        <v>7.304778603525278</v>
       </c>
       <c r="F2" t="n">
-        <v>0.0057304373364847</v>
+        <v>0.0073047786035252</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -1552,7 +1726,7 @@
         <v>0.875</v>
       </c>
       <c r="M2" t="n">
-        <v>3.166666666666667</v>
+        <v>4.166666666666667</v>
       </c>
     </row>
   </sheetData>
@@ -1663,10 +1837,10 @@
         <v>83579.11248</v>
       </c>
       <c r="G2" t="n">
-        <v>5.730437336484955</v>
+        <v>7.304778603525349</v>
       </c>
       <c r="H2" t="n">
-        <v>0.009794718810971201</v>
+        <v>0.0124856530482222</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -1674,7 +1848,7 @@
         </is>
       </c>
       <c r="J2" t="n">
-        <v>0.3028484098350931</v>
+        <v>0.3231071427947196</v>
       </c>
       <c r="K2" t="n">
         <v>0.033474721577948</v>
@@ -1749,7 +1923,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>-0.0162414039290576</v>
+        <v>-0.01362232159700749</v>
       </c>
       <c r="C2" t="n">
         <v>0.0244387654861391</v>
@@ -1758,11 +1932,11 @@
         <v>2</v>
       </c>
       <c r="E2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -1772,7 +1946,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>-0.004937674929030522</v>
+        <v>-0.002288498428524299</v>
       </c>
       <c r="C3" t="n">
         <v>0.0244387654861391</v>
@@ -1781,7 +1955,7 @@
         <v>1</v>
       </c>
       <c r="E3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="n">
@@ -1795,16 +1969,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.02145800519226237</v>
+        <v>0.01872943544870975</v>
       </c>
       <c r="C4" t="n">
-        <v>0.002514122551964482</v>
+        <v>0.006622656008078431</v>
       </c>
       <c r="D4" t="n">
         <v>1</v>
       </c>
       <c r="E4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="n">
@@ -1827,7 +2001,7 @@
         <v>1</v>
       </c>
       <c r="E5" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="n">
@@ -1850,7 +2024,7 @@
         <v>0</v>
       </c>
       <c r="E6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="n">
@@ -1864,7 +2038,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.001143949113574516</v>
+        <v>0.003809316856671741</v>
       </c>
       <c r="C7" t="n">
         <v>0.0244387654861391</v>
@@ -1873,7 +2047,7 @@
         <v>2</v>
       </c>
       <c r="E7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="n">
@@ -1887,7 +2061,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.006251824836175146</v>
+        <v>0.008930791390111326</v>
       </c>
       <c r="C8" t="n">
         <v>0.02443876548613899</v>
@@ -1896,7 +2070,7 @@
         <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="n">
@@ -1910,16 +2084,16 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>-0.01298101599849177</v>
+        <v>-0.01367192928729288</v>
       </c>
       <c r="C9" t="n">
-        <v>0.01637156673742368</v>
+        <v>0.01706010664070745</v>
       </c>
       <c r="D9" t="n">
         <v>4</v>
       </c>
       <c r="E9" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="n">
@@ -1933,7 +2107,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>-0.04884871046144057</v>
+        <v>-0.04631643928486684</v>
       </c>
       <c r="C10" t="n">
         <v>0.05407147927571376</v>
@@ -1942,7 +2116,7 @@
         <v>2</v>
       </c>
       <c r="E10" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="n">
@@ -1956,7 +2130,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.006007260149254456</v>
+        <v>0.005613788697409028</v>
       </c>
       <c r="C11" t="n">
         <v>0.0244387654861391</v>
@@ -1965,11 +2139,11 @@
         <v>1</v>
       </c>
       <c r="E11" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -1979,7 +2153,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>-0.03586740171412017</v>
+        <v>-0.03330057011131715</v>
       </c>
       <c r="C12" t="n">
         <v>0.0411614508549194</v>
@@ -1988,7 +2162,7 @@
         <v>2</v>
       </c>
       <c r="E12" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="n">
@@ -2002,7 +2176,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>-0.01920596579843037</v>
+        <v>-0.01814174437269811</v>
       </c>
       <c r="C13" t="n">
         <v>0.0244387654861391</v>
@@ -2011,11 +2185,11 @@
         <v>3</v>
       </c>
       <c r="E13" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -2025,7 +2199,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>-0.001346362927770017</v>
+        <v>0.001312374802339589</v>
       </c>
       <c r="C14" t="n">
         <v>0.02443876548613899</v>
@@ -2034,7 +2208,7 @@
         <v>2</v>
       </c>
       <c r="E14" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="n">
@@ -2048,7 +2222,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.009790405361835397</v>
+        <v>0.0124787927571981</v>
       </c>
       <c r="C15" t="n">
         <v>0.02443876548613899</v>
@@ -2057,7 +2231,7 @@
         <v>1</v>
       </c>
       <c r="E15" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="n">
@@ -2071,7 +2245,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>-0.002614961988878228</v>
+        <v>4.03983218109083e-05</v>
       </c>
       <c r="C16" t="n">
         <v>0.02443876548613921</v>
@@ -2080,7 +2254,7 @@
         <v>1</v>
       </c>
       <c r="E16" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="n">

</xml_diff>

<commit_message>
paper: actualización diaria 2026-10-06
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AtSxiX9NxnepDF7aXKR3KZ
</commit_message>
<xml_diff>
--- a/millonary/paper_state/semanal/diario.xlsx
+++ b/millonary/paper_state/semanal/diario.xlsx
@@ -442,7 +442,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-05 04:17:47.927392+00:00</t>
+          <t>2026-10-06 04:18:05.458761+00:00</t>
         </is>
       </c>
     </row>
@@ -473,7 +473,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1007.304778603525</v>
+        <v>1019.621773070849</v>
       </c>
     </row>
     <row r="6">
@@ -483,7 +483,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.007717453264318941</v>
+        <v>0.02003949378286962</v>
       </c>
     </row>
     <row r="7">
@@ -493,7 +493,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.007717453264318941</v>
+        <v>0.02003949378286962</v>
       </c>
     </row>
     <row r="8">
@@ -513,7 +513,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.01150055297838537</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -523,7 +523,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="11">
@@ -533,7 +533,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>26</v>
+        <v>32</v>
       </c>
     </row>
     <row r="12">
@@ -543,7 +543,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.5886740662762154</v>
+        <v>0.593729573052119</v>
       </c>
     </row>
     <row r="13">
@@ -553,7 +553,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>26</v>
+        <v>32</v>
       </c>
     </row>
     <row r="14">
@@ -640,7 +640,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>{"dias": 5, "estado": "insuficiente"}</t>
+          <t>{"dias": 6, "estado": "insuficiente"}</t>
         </is>
       </c>
     </row>
@@ -664,7 +664,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Mantener el objetivo del núcleo: 0.64× de exposición.</t>
+          <t>Mantener el objetivo del núcleo: 0.65× de exposición.</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>{"certificadas": [], "forward": {"S01 Parabolic SAR + EMA200": {"retorno": -0.013622321597007492, "caida_max": 0.024438765486139102, "ops": 2, "dias": 5, "sharpe": null, "posicion_actual": 0.0}, "S02 Ichimoku": {"retorno": -0.0022884984285242993, "caida_max": 0.024438765486139102, "ops": 1, "dias": 5, "sharpe": null, "posicion_actual": 1.0}, "S03 Bollinger + RSI (reversi\u00f3n)": {"retorno": 0.018729435448709753, "caida_max": 0.006622656008078431, "ops": 1, "dias": 5, "sharpe": null, "posicion_actual": -1.0}, "S04 Keltner ruptura": {"retorno": -0.02581271738866342, "caida_max": 0.02581271738866342, "ops": 1, "dias": 5, "sharpe": null, "posicion_actual": 0.0}, "S05 RSI(2) retroceso (largo)": {"retorno": 0.0, "caida_max": 0.0, "ops": 0, "dias": 5, "sharpe": null, "posicion_actual": 0.0}, "S06 Cruce SMA 7-25": {"retorno": 0.0038093168566717406, "caida_max": 0.024438765486139102, "ops": 2, "dias": 5, "sharpe": null, "posicion_actual": 1.0}, "S07 SMA 7-25 + filtro 200 (largo)": {"retorno": 0.008930791390111326, "caida_max": 0.02443876548613899, "ops": 1, "dias": 5, "sharpe": null, "posicion_actual": 1.0}, "S08 Canal 20 por tercios": {"retorno": -0.013671929287292883, "caida_max": 0.01706010664070745, "ops": 4, "dias": 5, "sharpe": null, "posicion_actual": 0.0}, "S09 Donchian 20/10": {"retorno": -0.04631643928486684, "caida_max": 0.05407147927571376, "ops": 2, "dias": 5, "sharpe": null, "posicion_actual": 1.0}, "S10 MACD + EMA200": {"retorno": 0.005613788697409028, "caida_max": 0.024438765486139102, "ops": 1, "dias": 5, "sharpe": null, "posicion_actual": 0.0}, "S11 Supertrend 10/3": {"retorno": -0.03330057011131715, "caida_max": 0.0411614508549194, "ops": 2, "dias": 5, "sharpe": null, "posicion_actual": 1.0}, "S12 Expansi\u00f3n de volatilidad": {"retorno": -0.01814174437269811, "caida_max": 0.024438765486139102, "ops": 3, "dias": 5, "sharpe": null, "posicion_actual": 0.0}, "S13 Retroceso a EMA20": {"retorno": 0.0013123748023395887, "caida_max": 0.02443876548613899, "ops": 2, "dias": 5, "sharpe": null, "posicion_actual": 1.0}, "S14 Momentum 90 d": {"retorno": 0.012478792757198098, "caida_max": 0.02443876548613899, "ops": 1, "dias": 5, "sharpe": null, "posicion_actual": 1.0}, "S15 RSI14 + EMA200": {"retorno": 4.03983218109083e-05, "caida_max": 0.024438765486139213, "ops": 1, "dias": 5, "sharpe": null, "posicion_actual": 1.0}}}</t>
+          <t>{"certificadas": [], "forward": {"S01 Parabolic SAR + EMA200": {"retorno": -0.014312785971889674, "caida_max": 0.024438765486139102, "ops": 2, "dias": 6, "sharpe": null, "posicion_actual": 0.0}, "S02 Ichimoku": {"retorno": -0.00193586779910071, "caida_max": 0.024438765486139102, "ops": 1, "dias": 6, "sharpe": null, "posicion_actual": 1.0}, "S03 Bollinger + RSI (reversi\u00f3n)": {"retorno": -0.002184153355806129, "caida_max": 0.025601434163612047, "ops": 1, "dias": 6, "sharpe": null, "posicion_actual": -1.0}, "S04 Keltner ruptura": {"retorno": -0.02581271738866342, "caida_max": 0.02581271738866342, "ops": 1, "dias": 6, "sharpe": null, "posicion_actual": 1.0}, "S05 RSI(2) retroceso (largo)": {"retorno": 0.0, "caida_max": 0.0, "ops": 0, "dias": 6, "sharpe": null, "posicion_actual": 0.0}, "S06 Cruce SMA 7-25": {"retorno": 0.02465993079551443, "caida_max": 0.024438765486139102, "ops": 2, "dias": 6, "sharpe": null, "posicion_actual": 1.0}, "S07 SMA 7-25 + filtro 200 (largo)": {"retorno": 0.0298877859796427, "caida_max": 0.02443876548613899, "ops": 1, "dias": 6, "sharpe": null, "posicion_actual": 1.0}, "S08 Canal 20 por tercios": {"retorno": -0.013671929287292883, "caida_max": 0.01706010664070745, "ops": 4, "dias": 6, "sharpe": null, "posicion_actual": 1.0}, "S09 Donchian 20/10": {"retorno": -0.026507011926133472, "caida_max": 0.05407147927571376, "ops": 2, "dias": 6, "sharpe": null, "posicion_actual": 1.0}, "S10 MACD + EMA200": {"retorno": 0.019914063781214075, "caida_max": 0.024438765486139102, "ops": 2, "dias": 6, "sharpe": null, "posicion_actual": 1.0}, "S11 Supertrend 10/3": {"retorno": -0.013220783772388223, "caida_max": 0.0411614508549194, "ops": 2, "dias": 6, "sharpe": null, "posicion_actual": 1.0}, "S12 Expansi\u00f3n de volatilidad": {"retorno": -0.01814174437269811, "caida_max": 0.024438765486139102, "ops": 3, "dias": 6, "sharpe": null, "posicion_actual": 0.0}, "S13 Retroceso a EMA20": {"retorno": 0.022111123537374544, "caida_max": 0.02443876548613899, "ops": 2, "dias": 6, "sharpe": null, "posicion_actual": 1.0}, "S14 Momentum 90 d": {"retorno": 0.03350948461723391, "caida_max": 0.02443876548613899, "ops": 1, "dias": 6, "sharpe": null, "posicion_actual": 1.0}, "S15 RSI14 + EMA200": {"retorno": 0.020812726211682175, "caida_max": 0.024438765486139213, "ops": 1, "dias": 6, "sharpe": null, "posicion_actual": 1.0}}}</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>{"n_pruebas": 75, "etapas": {"descartada (E1/E2)": 54, "E3 sombra": 21}, "adoptables": [], "top_forward": [], "ultima_actualizacion": "2026-10-05 04:17:47.927392+00:00"}</t>
+          <t>{"n_pruebas": 75, "etapas": {"descartada (E1/E2)": 54, "E3 sombra": 21}, "adoptables": [], "top_forward": [], "ultima_actualizacion": "2026-10-06 04:18:05.458761+00:00"}</t>
         </is>
       </c>
     </row>
@@ -703,7 +703,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I27"/>
+  <dimension ref="A1:I33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1506,6 +1506,180 @@
         <v>-0.0095138782269807</v>
       </c>
       <c r="I27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-10-04 04:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>1007.929878603525</v>
+      </c>
+      <c r="C28" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="D28" t="n">
+        <v>84799.89999999999</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0.5889291632295143</v>
+      </c>
+      <c r="F28" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="G28" t="n">
+        <v>0.6437160426996952</v>
+      </c>
+      <c r="H28" t="n">
+        <v>0</v>
+      </c>
+      <c r="I28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-10-04 08:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>1009.799494852815</v>
+      </c>
+      <c r="C29" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="D29" t="n">
+        <v>85070</v>
+      </c>
+      <c r="E29" t="n">
+        <v>0.5897111288283986</v>
+      </c>
+      <c r="F29" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="G29" t="n">
+        <v>0.6457946962132515</v>
+      </c>
+      <c r="H29" t="n">
+        <v>0.021083750710464</v>
+      </c>
+      <c r="I29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-10-04 12:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>1011.156794852815</v>
+      </c>
+      <c r="C30" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="D30" t="n">
+        <v>85263.89999999999</v>
+      </c>
+      <c r="E30" t="n">
+        <v>0.5902618694135146</v>
+      </c>
+      <c r="F30" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="G30" t="n">
+        <v>0.6480603366557198</v>
+      </c>
+      <c r="H30" t="n">
+        <v>0</v>
+      </c>
+      <c r="I30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-10-04 16:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>1010.718025972022</v>
+      </c>
+      <c r="C31" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="D31" t="n">
+        <v>85204.3</v>
+      </c>
+      <c r="E31" t="n">
+        <v>0.5901053356858901</v>
+      </c>
+      <c r="F31" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="G31" t="n">
+        <v>0.6503864077905364</v>
+      </c>
+      <c r="H31" t="n">
+        <v>0.0215688807929107</v>
+      </c>
+      <c r="I31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-10-04 20:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>1011.999725972022</v>
+      </c>
+      <c r="C32" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="D32" t="n">
+        <v>85387.39999999999</v>
+      </c>
+      <c r="E32" t="n">
+        <v>0.5906244682288823</v>
+      </c>
+      <c r="F32" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="G32" t="n">
+        <v>0.6526865013377076</v>
+      </c>
+      <c r="H32" t="n">
+        <v>0</v>
+      </c>
+      <c r="I32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-10-05 00:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>1019.621773070849</v>
+      </c>
+      <c r="C33" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="D33" t="n">
+        <v>86482.8</v>
+      </c>
+      <c r="E33" t="n">
+        <v>0.593729573052119</v>
+      </c>
+      <c r="F33" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="G33" t="n">
+        <v>0.6481483472075645</v>
+      </c>
+      <c r="H33" t="n">
+        <v>0.0457529011725506</v>
+      </c>
+      <c r="I33" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1700,10 +1874,10 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>7.304778603525278</v>
+        <v>19.62177307084925</v>
       </c>
       <c r="F2" t="n">
-        <v>0.0073047786035252</v>
+        <v>0.0196217730708492</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -1717,7 +1891,7 @@
         <v>83579.11248</v>
       </c>
       <c r="J2" t="n">
-        <v>0.033474721577948</v>
+        <v>0.0347417845660282</v>
       </c>
       <c r="K2" t="n">
         <v>-0.0038324465347324</v>
@@ -1726,7 +1900,7 @@
         <v>0.875</v>
       </c>
       <c r="M2" t="n">
-        <v>4.166666666666667</v>
+        <v>5.166666666666667</v>
       </c>
     </row>
   </sheetData>
@@ -1837,10 +2011,10 @@
         <v>83579.11248</v>
       </c>
       <c r="G2" t="n">
-        <v>7.304778603525349</v>
+        <v>19.6217730708494</v>
       </c>
       <c r="H2" t="n">
-        <v>0.0124856530482222</v>
+        <v>0.0335384087664671</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -1848,10 +2022,10 @@
         </is>
       </c>
       <c r="J2" t="n">
-        <v>0.3231071427947196</v>
+        <v>0.4115126754706451</v>
       </c>
       <c r="K2" t="n">
-        <v>0.033474721577948</v>
+        <v>0.0347417845660282</v>
       </c>
       <c r="L2" t="n">
         <v>-0.0038324465347324</v>
@@ -1923,7 +2097,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>-0.01362232159700749</v>
+        <v>-0.01431278597188967</v>
       </c>
       <c r="C2" t="n">
         <v>0.0244387654861391</v>
@@ -1932,7 +2106,7 @@
         <v>2</v>
       </c>
       <c r="E2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
@@ -1946,7 +2120,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>-0.002288498428524299</v>
+        <v>-0.00193586779910071</v>
       </c>
       <c r="C3" t="n">
         <v>0.0244387654861391</v>
@@ -1955,7 +2129,7 @@
         <v>1</v>
       </c>
       <c r="E3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="n">
@@ -1969,16 +2143,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.01872943544870975</v>
+        <v>-0.002184153355806129</v>
       </c>
       <c r="C4" t="n">
-        <v>0.006622656008078431</v>
+        <v>0.02560143416361205</v>
       </c>
       <c r="D4" t="n">
         <v>1</v>
       </c>
       <c r="E4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="n">
@@ -2001,11 +2175,11 @@
         <v>1</v>
       </c>
       <c r="E5" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -2024,7 +2198,7 @@
         <v>0</v>
       </c>
       <c r="E6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="n">
@@ -2038,7 +2212,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.003809316856671741</v>
+        <v>0.02465993079551443</v>
       </c>
       <c r="C7" t="n">
         <v>0.0244387654861391</v>
@@ -2047,7 +2221,7 @@
         <v>2</v>
       </c>
       <c r="E7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="n">
@@ -2061,7 +2235,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.008930791390111326</v>
+        <v>0.0298877859796427</v>
       </c>
       <c r="C8" t="n">
         <v>0.02443876548613899</v>
@@ -2070,7 +2244,7 @@
         <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="n">
@@ -2093,11 +2267,11 @@
         <v>4</v>
       </c>
       <c r="E9" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -2107,7 +2281,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>-0.04631643928486684</v>
+        <v>-0.02650701192613347</v>
       </c>
       <c r="C10" t="n">
         <v>0.05407147927571376</v>
@@ -2116,7 +2290,7 @@
         <v>2</v>
       </c>
       <c r="E10" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="n">
@@ -2130,20 +2304,20 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.005613788697409028</v>
+        <v>0.01991406378121408</v>
       </c>
       <c r="C11" t="n">
         <v>0.0244387654861391</v>
       </c>
       <c r="D11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E11" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
@@ -2153,7 +2327,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>-0.03330057011131715</v>
+        <v>-0.01322078377238822</v>
       </c>
       <c r="C12" t="n">
         <v>0.0411614508549194</v>
@@ -2162,7 +2336,7 @@
         <v>2</v>
       </c>
       <c r="E12" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="n">
@@ -2185,7 +2359,7 @@
         <v>3</v>
       </c>
       <c r="E13" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="n">
@@ -2199,7 +2373,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.001312374802339589</v>
+        <v>0.02211112353737454</v>
       </c>
       <c r="C14" t="n">
         <v>0.02443876548613899</v>
@@ -2208,7 +2382,7 @@
         <v>2</v>
       </c>
       <c r="E14" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="n">
@@ -2222,7 +2396,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.0124787927571981</v>
+        <v>0.03350948461723391</v>
       </c>
       <c r="C15" t="n">
         <v>0.02443876548613899</v>
@@ -2231,7 +2405,7 @@
         <v>1</v>
       </c>
       <c r="E15" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="n">
@@ -2245,7 +2419,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>4.03983218109083e-05</v>
+        <v>0.02081272621168218</v>
       </c>
       <c r="C16" t="n">
         <v>0.02443876548613921</v>
@@ -2254,7 +2428,7 @@
         <v>1</v>
       </c>
       <c r="E16" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="n">

</xml_diff>

<commit_message>
paper: actualización diaria 2026-10-07
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AtSxiX9NxnepDF7aXKR3KZ
</commit_message>
<xml_diff>
--- a/millonary/paper_state/semanal/diario.xlsx
+++ b/millonary/paper_state/semanal/diario.xlsx
@@ -442,7 +442,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-06 04:18:05.458761+00:00</t>
+          <t>2026-10-07 04:18:06.319742+00:00</t>
         </is>
       </c>
     </row>
@@ -473,7 +473,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1019.621773070849</v>
+        <v>1014.263736395998</v>
       </c>
     </row>
     <row r="6">
@@ -483,7 +483,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.02003949378286962</v>
+        <v>0.01467926201670777</v>
       </c>
     </row>
     <row r="7">
@@ -493,7 +493,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.02003949378286962</v>
+        <v>0.01682088983809904</v>
       </c>
     </row>
     <row r="8">
@@ -513,7 +513,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0</v>
+        <v>0.00525492571496744</v>
       </c>
     </row>
     <row r="10">
@@ -523,7 +523,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11">
@@ -533,7 +533,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>32</v>
+        <v>38</v>
       </c>
     </row>
     <row r="12">
@@ -543,7 +543,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.593729573052119</v>
+        <v>0.5915822270567055</v>
       </c>
     </row>
     <row r="13">
@@ -553,7 +553,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>32</v>
+        <v>35</v>
       </c>
     </row>
     <row r="14">
@@ -573,7 +573,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -593,7 +593,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0.29252689368</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -640,7 +640,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>{"dias": 6, "estado": "insuficiente"}</t>
+          <t>{"dias": 7, "estado": "insuficiente"}</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>{"certificadas": [], "forward": {"S01 Parabolic SAR + EMA200": {"retorno": -0.014312785971889674, "caida_max": 0.024438765486139102, "ops": 2, "dias": 6, "sharpe": null, "posicion_actual": 0.0}, "S02 Ichimoku": {"retorno": -0.00193586779910071, "caida_max": 0.024438765486139102, "ops": 1, "dias": 6, "sharpe": null, "posicion_actual": 1.0}, "S03 Bollinger + RSI (reversi\u00f3n)": {"retorno": -0.002184153355806129, "caida_max": 0.025601434163612047, "ops": 1, "dias": 6, "sharpe": null, "posicion_actual": -1.0}, "S04 Keltner ruptura": {"retorno": -0.02581271738866342, "caida_max": 0.02581271738866342, "ops": 1, "dias": 6, "sharpe": null, "posicion_actual": 1.0}, "S05 RSI(2) retroceso (largo)": {"retorno": 0.0, "caida_max": 0.0, "ops": 0, "dias": 6, "sharpe": null, "posicion_actual": 0.0}, "S06 Cruce SMA 7-25": {"retorno": 0.02465993079551443, "caida_max": 0.024438765486139102, "ops": 2, "dias": 6, "sharpe": null, "posicion_actual": 1.0}, "S07 SMA 7-25 + filtro 200 (largo)": {"retorno": 0.0298877859796427, "caida_max": 0.02443876548613899, "ops": 1, "dias": 6, "sharpe": null, "posicion_actual": 1.0}, "S08 Canal 20 por tercios": {"retorno": -0.013671929287292883, "caida_max": 0.01706010664070745, "ops": 4, "dias": 6, "sharpe": null, "posicion_actual": 1.0}, "S09 Donchian 20/10": {"retorno": -0.026507011926133472, "caida_max": 0.05407147927571376, "ops": 2, "dias": 6, "sharpe": null, "posicion_actual": 1.0}, "S10 MACD + EMA200": {"retorno": 0.019914063781214075, "caida_max": 0.024438765486139102, "ops": 2, "dias": 6, "sharpe": null, "posicion_actual": 1.0}, "S11 Supertrend 10/3": {"retorno": -0.013220783772388223, "caida_max": 0.0411614508549194, "ops": 2, "dias": 6, "sharpe": null, "posicion_actual": 1.0}, "S12 Expansi\u00f3n de volatilidad": {"retorno": -0.01814174437269811, "caida_max": 0.024438765486139102, "ops": 3, "dias": 6, "sharpe": null, "posicion_actual": 0.0}, "S13 Retroceso a EMA20": {"retorno": 0.022111123537374544, "caida_max": 0.02443876548613899, "ops": 2, "dias": 6, "sharpe": null, "posicion_actual": 1.0}, "S14 Momentum 90 d": {"retorno": 0.03350948461723391, "caida_max": 0.02443876548613899, "ops": 1, "dias": 6, "sharpe": null, "posicion_actual": 1.0}, "S15 RSI14 + EMA200": {"retorno": 0.020812726211682175, "caida_max": 0.024438765486139213, "ops": 1, "dias": 6, "sharpe": null, "posicion_actual": 1.0}}}</t>
+          <t>{"certificadas": [], "forward": {"S01 Parabolic SAR + EMA200": {"retorno": -0.01881068660924845, "caida_max": 0.030221347464636117, "ops": 3, "dias": 7, "sharpe": null, "posicion_actual": 1.0}, "S02 Ichimoku": {"retorno": -0.011464760775629523, "caida_max": 0.03405983944279534, "ops": 2, "dias": 7, "sharpe": null, "posicion_actual": 1.0}, "S03 Bollinger + RSI (reversi\u00f3n)": {"retorno": 0.011763122737633136, "caida_max": 0.025601434163612047, "ops": 1, "dias": 7, "sharpe": null, "posicion_actual": 0.0}, "S04 Keltner ruptura": {"retorno": -0.041404541369365444, "caida_max": 0.041404541369365444, "ops": 2, "dias": 7, "sharpe": null, "posicion_actual": 0.0}, "S05 RSI(2) retroceso (largo)": {"retorno": 0.0, "caida_max": 0.0, "ops": 0, "dias": 7, "sharpe": null, "posicion_actual": 0.0}, "S06 Cruce SMA 7-25": {"retorno": 0.015591605846117185, "caida_max": 0.024438765486139102, "ops": 2, "dias": 7, "sharpe": null, "posicion_actual": 1.0}, "S07 SMA 7-25 + filtro 200 (largo)": {"retorno": 0.02077319408042788, "caida_max": 0.02443876548613899, "ops": 1, "dias": 7, "sharpe": null, "posicion_actual": 1.0}, "S08 Canal 20 por tercios": {"retorno": -0.032702207781938775, "caida_max": 0.036025013419248686, "ops": 6, "dias": 7, "sharpe": null, "posicion_actual": 0.0}, "S09 Donchian 20/10": {"retorno": -0.035122505209802535, "caida_max": 0.05407147927571376, "ops": 2, "dias": 7, "sharpe": null, "posicion_actual": 1.0}, "S10 MACD + EMA200": {"retorno": 0.010887740146554359, "caida_max": 0.024438765486139102, "ops": 2, "dias": 7, "sharpe": null, "posicion_actual": 1.0}, "S11 Supertrend 10/3": {"retorno": -0.02195386127168708, "caida_max": 0.0411614508549194, "ops": 2, "dias": 7, "sharpe": null, "posicion_actual": 1.0}, "S12 Expansi\u00f3n de volatilidad": {"retorno": -0.01814174437269811, "caida_max": 0.024438765486139102, "ops": 3, "dias": 7, "sharpe": null, "posicion_actual": 0.0}, "S13 Retroceso a EMA20": {"retorno": 0.01306535574255685, "caida_max": 0.02443876548613899, "ops": 2, "dias": 7, "sharpe": null, "posicion_actual": 1.0}, "S14 Momentum 90 d": {"retorno": 0.02436284038618952, "caida_max": 0.02443876548613899, "ops": 1, "dias": 7, "sharpe": null, "posicion_actual": 1.0}, "S15 RSI14 + EMA200": {"retorno": 0.011778449340349217, "caida_max": 0.024438765486139213, "ops": 1, "dias": 7, "sharpe": null, "posicion_actual": 1.0}}}</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>{"n_pruebas": 75, "etapas": {"descartada (E1/E2)": 54, "E3 sombra": 21}, "adoptables": [], "top_forward": [], "ultima_actualizacion": "2026-10-06 04:18:05.458761+00:00"}</t>
+          <t>{"n_pruebas": 75, "etapas": {"descartada (E1/E2)": 54, "E3 sombra": 21}, "adoptables": [], "top_forward": [], "ultima_actualizacion": "2026-10-07 04:18:06.319742+00:00"}</t>
         </is>
       </c>
     </row>
@@ -703,7 +703,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I33"/>
+  <dimension ref="A1:I39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1680,6 +1680,180 @@
         <v>0.0457529011725506</v>
       </c>
       <c r="I33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-10-05 04:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>1016.593573070849</v>
+      </c>
+      <c r="C34" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="D34" t="n">
+        <v>86050.2</v>
+      </c>
+      <c r="E34" t="n">
+        <v>0.5925193862680661</v>
+      </c>
+      <c r="F34" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="G34" t="n">
+        <v>0.6490535534587727</v>
+      </c>
+      <c r="H34" t="n">
+        <v>0</v>
+      </c>
+      <c r="I34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-10-05 08:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>1017.767599123715</v>
+      </c>
+      <c r="C35" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="D35" t="n">
+        <v>86221.60000000001</v>
+      </c>
+      <c r="E35" t="n">
+        <v>0.5930147516187879</v>
+      </c>
+      <c r="F35" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="G35" t="n">
+        <v>0.6513785718993643</v>
+      </c>
+      <c r="H35" t="n">
+        <v>0.0257739471342342</v>
+      </c>
+      <c r="I35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-10-05 12:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>1017.373499123715</v>
+      </c>
+      <c r="C36" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="D36" t="n">
+        <v>86165.3</v>
+      </c>
+      <c r="E36" t="n">
+        <v>0.5928570977320639</v>
+      </c>
+      <c r="F36" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="G36" t="n">
+        <v>0.6537140348237341</v>
+      </c>
+      <c r="H36" t="n">
+        <v>0</v>
+      </c>
+      <c r="I36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-10-05 16:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>1010.769175639032</v>
+      </c>
+      <c r="C37" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="D37" t="n">
+        <v>85220.3</v>
+      </c>
+      <c r="E37" t="n">
+        <v>0.5901862802878332</v>
+      </c>
+      <c r="F37" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="G37" t="n">
+        <v>0.6498092848537009</v>
+      </c>
+      <c r="H37" t="n">
+        <v>-0.0106765153173289</v>
+      </c>
+      <c r="I37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-10-05 20:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>1014.065475639032</v>
+      </c>
+      <c r="C38" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="D38" t="n">
+        <v>85691.2</v>
+      </c>
+      <c r="E38" t="n">
+        <v>0.5915184121833953</v>
+      </c>
+      <c r="F38" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="G38" t="n">
+        <v>0.6510753136706323</v>
+      </c>
+      <c r="H38" t="n">
+        <v>0</v>
+      </c>
+      <c r="I38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-10-06 00:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>1014.263736395998</v>
+      </c>
+      <c r="C39" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="D39" t="n">
+        <v>85717.2</v>
+      </c>
+      <c r="E39" t="n">
+        <v>0.5915822270567055</v>
+      </c>
+      <c r="F39" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="G39" t="n">
+        <v>0.6534869230223079</v>
+      </c>
+      <c r="H39" t="n">
+        <v>-0.0162607569659628</v>
+      </c>
+      <c r="I39" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1874,10 +2048,10 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>19.62177307084925</v>
+        <v>14.26373639599831</v>
       </c>
       <c r="F2" t="n">
-        <v>0.0196217730708492</v>
+        <v>0.0142637363959983</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -1900,7 +2074,7 @@
         <v>0.875</v>
       </c>
       <c r="M2" t="n">
-        <v>5.166666666666667</v>
+        <v>6.166666666666667</v>
       </c>
     </row>
   </sheetData>
@@ -2011,10 +2185,10 @@
         <v>83579.11248</v>
       </c>
       <c r="G2" t="n">
-        <v>19.6217730708494</v>
+        <v>14.26373639599842</v>
       </c>
       <c r="H2" t="n">
-        <v>0.0335384087664671</v>
+        <v>0.0243802137584002</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -2022,7 +2196,7 @@
         </is>
       </c>
       <c r="J2" t="n">
-        <v>0.4115126754706451</v>
+        <v>0.4103493503215876</v>
       </c>
       <c r="K2" t="n">
         <v>0.0347417845660282</v>
@@ -2097,20 +2271,20 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>-0.01431278597188967</v>
+        <v>-0.01881068660924845</v>
       </c>
       <c r="C2" t="n">
-        <v>0.0244387654861391</v>
+        <v>0.03022134746463612</v>
       </c>
       <c r="D2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -2120,16 +2294,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>-0.00193586779910071</v>
+        <v>-0.01146476077562952</v>
       </c>
       <c r="C3" t="n">
-        <v>0.0244387654861391</v>
+        <v>0.03405983944279534</v>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E3" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="n">
@@ -2143,7 +2317,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>-0.002184153355806129</v>
+        <v>0.01176312273763314</v>
       </c>
       <c r="C4" t="n">
         <v>0.02560143416361205</v>
@@ -2152,11 +2326,11 @@
         <v>1</v>
       </c>
       <c r="E4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -2166,20 +2340,20 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>-0.02581271738866342</v>
+        <v>-0.04140454136936544</v>
       </c>
       <c r="C5" t="n">
-        <v>0.02581271738866342</v>
+        <v>0.04140454136936544</v>
       </c>
       <c r="D5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E5" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -2198,7 +2372,7 @@
         <v>0</v>
       </c>
       <c r="E6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="n">
@@ -2212,7 +2386,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.02465993079551443</v>
+        <v>0.01559160584611718</v>
       </c>
       <c r="C7" t="n">
         <v>0.0244387654861391</v>
@@ -2221,7 +2395,7 @@
         <v>2</v>
       </c>
       <c r="E7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="n">
@@ -2235,7 +2409,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.0298877859796427</v>
+        <v>0.02077319408042788</v>
       </c>
       <c r="C8" t="n">
         <v>0.02443876548613899</v>
@@ -2244,7 +2418,7 @@
         <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="n">
@@ -2258,20 +2432,20 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>-0.01367192928729288</v>
+        <v>-0.03270220778193877</v>
       </c>
       <c r="C9" t="n">
-        <v>0.01706010664070745</v>
+        <v>0.03602501341924869</v>
       </c>
       <c r="D9" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E9" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -2281,7 +2455,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>-0.02650701192613347</v>
+        <v>-0.03512250520980253</v>
       </c>
       <c r="C10" t="n">
         <v>0.05407147927571376</v>
@@ -2290,7 +2464,7 @@
         <v>2</v>
       </c>
       <c r="E10" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="n">
@@ -2304,7 +2478,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.01991406378121408</v>
+        <v>0.01088774014655436</v>
       </c>
       <c r="C11" t="n">
         <v>0.0244387654861391</v>
@@ -2313,7 +2487,7 @@
         <v>2</v>
       </c>
       <c r="E11" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="n">
@@ -2327,7 +2501,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>-0.01322078377238822</v>
+        <v>-0.02195386127168708</v>
       </c>
       <c r="C12" t="n">
         <v>0.0411614508549194</v>
@@ -2336,7 +2510,7 @@
         <v>2</v>
       </c>
       <c r="E12" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="n">
@@ -2359,7 +2533,7 @@
         <v>3</v>
       </c>
       <c r="E13" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="n">
@@ -2373,7 +2547,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.02211112353737454</v>
+        <v>0.01306535574255685</v>
       </c>
       <c r="C14" t="n">
         <v>0.02443876548613899</v>
@@ -2382,7 +2556,7 @@
         <v>2</v>
       </c>
       <c r="E14" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="n">
@@ -2396,7 +2570,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.03350948461723391</v>
+        <v>0.02436284038618952</v>
       </c>
       <c r="C15" t="n">
         <v>0.02443876548613899</v>
@@ -2405,7 +2579,7 @@
         <v>1</v>
       </c>
       <c r="E15" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="n">
@@ -2419,7 +2593,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.02081272621168218</v>
+        <v>0.01177844934034922</v>
       </c>
       <c r="C16" t="n">
         <v>0.02443876548613921</v>
@@ -2428,7 +2602,7 @@
         <v>1</v>
       </c>
       <c r="E16" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="n">

</xml_diff>

<commit_message>
paper: actualización diaria 2026-10-08
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AtSxiX9NxnepDF7aXKR3KZ
</commit_message>
<xml_diff>
--- a/millonary/paper_state/semanal/diario.xlsx
+++ b/millonary/paper_state/semanal/diario.xlsx
@@ -442,7 +442,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-07 04:18:06.319742+00:00</t>
+          <t>2026-10-08 04:17:48.009895+00:00</t>
         </is>
       </c>
     </row>
@@ -473,7 +473,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1014.263736395998</v>
+        <v>1012.797648024174</v>
       </c>
     </row>
     <row r="6">
@@ -483,7 +483,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.01467926201670777</v>
+        <v>0.01321257301483136</v>
       </c>
     </row>
     <row r="7">
@@ -493,7 +493,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.01682088983809904</v>
+        <v>0.01221999933681284</v>
       </c>
     </row>
     <row r="8">
@@ -513,7 +513,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.00525492571496744</v>
+        <v>0.006692800435324719</v>
       </c>
     </row>
     <row r="10">
@@ -523,7 +523,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="11">
@@ -533,7 +533,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>38</v>
+        <v>44</v>
       </c>
     </row>
     <row r="12">
@@ -543,7 +543,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.5915822270567055</v>
+        <v>0.5909892278755701</v>
       </c>
     </row>
     <row r="13">
@@ -640,7 +640,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>{"dias": 7, "estado": "insuficiente"}</t>
+          <t>{"dias": 8, "estado": "insuficiente"}</t>
         </is>
       </c>
     </row>
@@ -664,7 +664,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Mantener el objetivo del núcleo: 0.65× de exposición.</t>
+          <t>Mantener el objetivo del núcleo: 0.66× de exposición.</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>{"certificadas": [], "forward": {"S01 Parabolic SAR + EMA200": {"retorno": -0.01881068660924845, "caida_max": 0.030221347464636117, "ops": 3, "dias": 7, "sharpe": null, "posicion_actual": 1.0}, "S02 Ichimoku": {"retorno": -0.011464760775629523, "caida_max": 0.03405983944279534, "ops": 2, "dias": 7, "sharpe": null, "posicion_actual": 1.0}, "S03 Bollinger + RSI (reversi\u00f3n)": {"retorno": 0.011763122737633136, "caida_max": 0.025601434163612047, "ops": 1, "dias": 7, "sharpe": null, "posicion_actual": 0.0}, "S04 Keltner ruptura": {"retorno": -0.041404541369365444, "caida_max": 0.041404541369365444, "ops": 2, "dias": 7, "sharpe": null, "posicion_actual": 0.0}, "S05 RSI(2) retroceso (largo)": {"retorno": 0.0, "caida_max": 0.0, "ops": 0, "dias": 7, "sharpe": null, "posicion_actual": 0.0}, "S06 Cruce SMA 7-25": {"retorno": 0.015591605846117185, "caida_max": 0.024438765486139102, "ops": 2, "dias": 7, "sharpe": null, "posicion_actual": 1.0}, "S07 SMA 7-25 + filtro 200 (largo)": {"retorno": 0.02077319408042788, "caida_max": 0.02443876548613899, "ops": 1, "dias": 7, "sharpe": null, "posicion_actual": 1.0}, "S08 Canal 20 por tercios": {"retorno": -0.032702207781938775, "caida_max": 0.036025013419248686, "ops": 6, "dias": 7, "sharpe": null, "posicion_actual": 0.0}, "S09 Donchian 20/10": {"retorno": -0.035122505209802535, "caida_max": 0.05407147927571376, "ops": 2, "dias": 7, "sharpe": null, "posicion_actual": 1.0}, "S10 MACD + EMA200": {"retorno": 0.010887740146554359, "caida_max": 0.024438765486139102, "ops": 2, "dias": 7, "sharpe": null, "posicion_actual": 1.0}, "S11 Supertrend 10/3": {"retorno": -0.02195386127168708, "caida_max": 0.0411614508549194, "ops": 2, "dias": 7, "sharpe": null, "posicion_actual": 1.0}, "S12 Expansi\u00f3n de volatilidad": {"retorno": -0.01814174437269811, "caida_max": 0.024438765486139102, "ops": 3, "dias": 7, "sharpe": null, "posicion_actual": 0.0}, "S13 Retroceso a EMA20": {"retorno": 0.01306535574255685, "caida_max": 0.02443876548613899, "ops": 2, "dias": 7, "sharpe": null, "posicion_actual": 1.0}, "S14 Momentum 90 d": {"retorno": 0.02436284038618952, "caida_max": 0.02443876548613899, "ops": 1, "dias": 7, "sharpe": null, "posicion_actual": 1.0}, "S15 RSI14 + EMA200": {"retorno": 0.011778449340349217, "caida_max": 0.024438765486139213, "ops": 1, "dias": 7, "sharpe": null, "posicion_actual": 1.0}}}</t>
+          <t>{"certificadas": [], "forward": {"S01 Parabolic SAR + EMA200": {"retorno": -0.021208204502223826, "caida_max": 0.030221347464636117, "ops": 3, "dias": 8, "sharpe": null, "posicion_actual": 1.0}, "S02 Ichimoku": {"retorno": -0.013880228302163289, "caida_max": 0.03405983944279534, "ops": 2, "dias": 8, "sharpe": null, "posicion_actual": 1.0}, "S03 Bollinger + RSI (reversi\u00f3n)": {"retorno": 0.011763122737633136, "caida_max": 0.025601434163612047, "ops": 1, "dias": 8, "sharpe": null, "posicion_actual": 0.0}, "S04 Keltner ruptura": {"retorno": -0.041404541369365444, "caida_max": 0.041404541369365444, "ops": 2, "dias": 8, "sharpe": null, "posicion_actual": 0.0}, "S05 RSI(2) retroceso (largo)": {"retorno": 0.0, "caida_max": 0.0, "ops": 0, "dias": 8, "sharpe": null, "posicion_actual": 0.0}, "S06 Cruce SMA 7-25": {"retorno": 0.013110026589452373, "caida_max": 0.024438765486139102, "ops": 2, "dias": 8, "sharpe": null, "posicion_actual": 1.0}, "S07 SMA 7-25 + filtro 200 (largo)": {"retorno": 0.01827895370899535, "caida_max": 0.02443876548613899, "ops": 1, "dias": 8, "sharpe": null, "posicion_actual": 1.0}, "S08 Canal 20 por tercios": {"retorno": -0.04008285523508004, "caida_max": 0.04338030729755338, "ops": 7, "dias": 8, "sharpe": null, "posicion_actual": 0.0}, "S09 Donchian 20/10": {"retorno": -0.03748016547649924, "caida_max": 0.05407147927571376, "ops": 2, "dias": 8, "sharpe": null, "posicion_actual": 1.0}, "S10 MACD + EMA200": {"retorno": 0.0073257834870295024, "caida_max": 0.024438765486139102, "ops": 2, "dias": 8, "sharpe": null, "posicion_actual": 0.0}, "S11 Supertrend 10/3": {"retorno": -0.024343698875659014, "caida_max": 0.0411614508549194, "ops": 2, "dias": 8, "sharpe": null, "posicion_actual": 1.0}, "S12 Expansi\u00f3n de volatilidad": {"retorno": -0.01814174437269811, "caida_max": 0.024438765486139102, "ops": 3, "dias": 8, "sharpe": null, "posicion_actual": 0.0}, "S13 Retroceso a EMA20": {"retorno": 0.010589949331175408, "caida_max": 0.02443876548613899, "ops": 2, "dias": 8, "sharpe": null, "posicion_actual": 1.0}, "S14 Momentum 90 d": {"retorno": 0.02185982878057202, "caida_max": 0.02443876548613899, "ops": 1, "dias": 8, "sharpe": null, "posicion_actual": 1.0}, "S15 RSI14 + EMA200": {"retorno": 0.009306187460898618, "caida_max": 0.024438765486139213, "ops": 1, "dias": 8, "sharpe": null, "posicion_actual": 1.0}}}</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>{"n_pruebas": 75, "etapas": {"descartada (E1/E2)": 54, "E3 sombra": 21}, "adoptables": [], "top_forward": [], "ultima_actualizacion": "2026-10-07 04:18:06.319742+00:00"}</t>
+          <t>{"n_pruebas": 75, "etapas": {"descartada (E1/E2)": 54, "E3 sombra": 21}, "adoptables": [], "top_forward": [], "ultima_actualizacion": "2026-10-08 04:17:48.009895+00:00"}</t>
         </is>
       </c>
     </row>
@@ -703,7 +703,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I39"/>
+  <dimension ref="A1:I45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1854,6 +1854,180 @@
         <v>-0.0162607569659628</v>
       </c>
       <c r="I39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-10-06 04:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>1012.568336395998</v>
+      </c>
+      <c r="C40" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="D40" t="n">
+        <v>85475</v>
+      </c>
+      <c r="E40" t="n">
+        <v>0.590898390255416</v>
+      </c>
+      <c r="F40" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="G40" t="n">
+        <v>0.6553541407907832</v>
+      </c>
+      <c r="H40" t="n">
+        <v>0</v>
+      </c>
+      <c r="I40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-10-06 08:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>1012.839255141761</v>
+      </c>
+      <c r="C41" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="D41" t="n">
+        <v>85512.39999999999</v>
+      </c>
+      <c r="E41" t="n">
+        <v>0.5909988154203395</v>
+      </c>
+      <c r="F41" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="G41" t="n">
+        <v>0.6577849568532629</v>
+      </c>
+      <c r="H41" t="n">
+        <v>-0.009118745763011299</v>
+      </c>
+      <c r="I41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-10-06 12:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>1017.729455141761</v>
+      </c>
+      <c r="C42" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="D42" t="n">
+        <v>86211</v>
+      </c>
+      <c r="E42" t="n">
+        <v>0.5929640701181638</v>
+      </c>
+      <c r="F42" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="G42" t="n">
+        <v>0.6574492947035508</v>
+      </c>
+      <c r="H42" t="n">
+        <v>0</v>
+      </c>
+      <c r="I42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-10-06 16:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>1013.966831545016</v>
+      </c>
+      <c r="C43" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="D43" t="n">
+        <v>85675.10000000001</v>
+      </c>
+      <c r="E43" t="n">
+        <v>0.591464810625193</v>
+      </c>
+      <c r="F43" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="G43" t="n">
+        <v>0.6576314157192603</v>
+      </c>
+      <c r="H43" t="n">
+        <v>0.0113235967448677</v>
+      </c>
+      <c r="I43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-10-06 20:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>1013.224131545016</v>
+      </c>
+      <c r="C44" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="D44" t="n">
+        <v>85569</v>
+      </c>
+      <c r="E44" t="n">
+        <v>0.5911653516252519</v>
+      </c>
+      <c r="F44" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="G44" t="n">
+        <v>0.6599112862854334</v>
+      </c>
+      <c r="H44" t="n">
+        <v>0</v>
+      </c>
+      <c r="I44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-10-07 00:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>1012.797648024174</v>
+      </c>
+      <c r="C45" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="D45" t="n">
+        <v>85507.5</v>
+      </c>
+      <c r="E45" t="n">
+        <v>0.5909892278755701</v>
+      </c>
+      <c r="F45" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="G45" t="n">
+        <v>0.6622789367800357</v>
+      </c>
+      <c r="H45" t="n">
+        <v>-0.0040164791576372</v>
+      </c>
+      <c r="I45" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2048,10 +2222,10 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>14.26373639599831</v>
+        <v>12.79764802417412</v>
       </c>
       <c r="F2" t="n">
-        <v>0.0142637363959983</v>
+        <v>0.0127976480241741</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -2074,7 +2248,7 @@
         <v>0.875</v>
       </c>
       <c r="M2" t="n">
-        <v>6.166666666666667</v>
+        <v>7.166666666666667</v>
       </c>
     </row>
   </sheetData>
@@ -2185,10 +2359,10 @@
         <v>83579.11248</v>
       </c>
       <c r="G2" t="n">
-        <v>14.26373639599842</v>
+        <v>12.79764802417422</v>
       </c>
       <c r="H2" t="n">
-        <v>0.0243802137584002</v>
+        <v>0.0218743101927814</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -2196,7 +2370,7 @@
         </is>
       </c>
       <c r="J2" t="n">
-        <v>0.4103493503215876</v>
+        <v>0.4085377221458068</v>
       </c>
       <c r="K2" t="n">
         <v>0.0347417845660282</v>
@@ -2271,7 +2445,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>-0.01881068660924845</v>
+        <v>-0.02120820450222383</v>
       </c>
       <c r="C2" t="n">
         <v>0.03022134746463612</v>
@@ -2280,7 +2454,7 @@
         <v>3</v>
       </c>
       <c r="E2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
@@ -2294,7 +2468,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>-0.01146476077562952</v>
+        <v>-0.01388022830216329</v>
       </c>
       <c r="C3" t="n">
         <v>0.03405983944279534</v>
@@ -2303,7 +2477,7 @@
         <v>2</v>
       </c>
       <c r="E3" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="n">
@@ -2326,7 +2500,7 @@
         <v>1</v>
       </c>
       <c r="E4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="n">
@@ -2349,7 +2523,7 @@
         <v>2</v>
       </c>
       <c r="E5" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="n">
@@ -2372,7 +2546,7 @@
         <v>0</v>
       </c>
       <c r="E6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="n">
@@ -2386,7 +2560,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.01559160584611718</v>
+        <v>0.01311002658945237</v>
       </c>
       <c r="C7" t="n">
         <v>0.0244387654861391</v>
@@ -2395,7 +2569,7 @@
         <v>2</v>
       </c>
       <c r="E7" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="n">
@@ -2409,7 +2583,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.02077319408042788</v>
+        <v>0.01827895370899535</v>
       </c>
       <c r="C8" t="n">
         <v>0.02443876548613899</v>
@@ -2418,7 +2592,7 @@
         <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="n">
@@ -2432,16 +2606,16 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>-0.03270220778193877</v>
+        <v>-0.04008285523508004</v>
       </c>
       <c r="C9" t="n">
-        <v>0.03602501341924869</v>
+        <v>0.04338030729755338</v>
       </c>
       <c r="D9" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E9" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="n">
@@ -2455,7 +2629,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>-0.03512250520980253</v>
+        <v>-0.03748016547649924</v>
       </c>
       <c r="C10" t="n">
         <v>0.05407147927571376</v>
@@ -2464,7 +2638,7 @@
         <v>2</v>
       </c>
       <c r="E10" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="n">
@@ -2478,7 +2652,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.01088774014655436</v>
+        <v>0.007325783487029502</v>
       </c>
       <c r="C11" t="n">
         <v>0.0244387654861391</v>
@@ -2487,11 +2661,11 @@
         <v>2</v>
       </c>
       <c r="E11" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -2501,7 +2675,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>-0.02195386127168708</v>
+        <v>-0.02434369887565901</v>
       </c>
       <c r="C12" t="n">
         <v>0.0411614508549194</v>
@@ -2510,7 +2684,7 @@
         <v>2</v>
       </c>
       <c r="E12" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="n">
@@ -2533,7 +2707,7 @@
         <v>3</v>
       </c>
       <c r="E13" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="n">
@@ -2547,7 +2721,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.01306535574255685</v>
+        <v>0.01058994933117541</v>
       </c>
       <c r="C14" t="n">
         <v>0.02443876548613899</v>
@@ -2556,7 +2730,7 @@
         <v>2</v>
       </c>
       <c r="E14" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="n">
@@ -2570,7 +2744,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.02436284038618952</v>
+        <v>0.02185982878057202</v>
       </c>
       <c r="C15" t="n">
         <v>0.02443876548613899</v>
@@ -2579,7 +2753,7 @@
         <v>1</v>
       </c>
       <c r="E15" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="n">
@@ -2593,7 +2767,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.01177844934034922</v>
+        <v>0.009306187460898618</v>
       </c>
       <c r="C16" t="n">
         <v>0.02443876548613921</v>
@@ -2602,7 +2776,7 @@
         <v>1</v>
       </c>
       <c r="E16" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="n">

</xml_diff>

<commit_message>
paper: actualización diaria 2026-10-09
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AtSxiX9NxnepDF7aXKR3KZ
</commit_message>
<xml_diff>
--- a/millonary/paper_state/semanal/diario.xlsx
+++ b/millonary/paper_state/semanal/diario.xlsx
@@ -442,7 +442,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-08 04:17:48.009895+00:00</t>
+          <t>2026-10-09 04:17:55.538927+00:00</t>
         </is>
       </c>
     </row>
@@ -473,7 +473,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1012.797648024174</v>
+        <v>996.8922903113749</v>
       </c>
     </row>
     <row r="6">
@@ -483,7 +483,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.01321257301483136</v>
+        <v>-0.002699300837112895</v>
       </c>
     </row>
     <row r="7">
@@ -493,7 +493,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.01221999933681284</v>
+        <v>-0.01568942775918525</v>
       </c>
     </row>
     <row r="8">
@@ -503,7 +503,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.01450074688943914</v>
+        <v>0.02229207276637357</v>
       </c>
     </row>
     <row r="9">
@@ -513,7 +513,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.006692800435324719</v>
+        <v>0.02229207276637357</v>
       </c>
     </row>
     <row r="10">
@@ -523,7 +523,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="11">
@@ -533,7 +533,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>44</v>
+        <v>50</v>
       </c>
     </row>
     <row r="12">
@@ -543,7 +543,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.5909892278755701</v>
+        <v>0.7518737051982671</v>
       </c>
     </row>
     <row r="13">
@@ -563,7 +563,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15">
@@ -573,7 +573,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.29252689368</v>
+        <v>0.37594287354</v>
       </c>
     </row>
     <row r="17">
@@ -593,7 +593,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0</v>
+        <v>0.08341597986</v>
       </c>
     </row>
     <row r="18">
@@ -616,7 +616,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>{"cerrados": 0, "ganan": 0, "pierden": 0, "abiertos": 1}</t>
+          <t>{"cerrados": 0, "ganan": 0, "pierden": 0, "abiertos": 2}</t>
         </is>
       </c>
     </row>
@@ -640,7 +640,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>{"dias": 8, "estado": "insuficiente"}</t>
+          <t>{"dias": 9, "estado": "insuficiente"}</t>
         </is>
       </c>
     </row>
@@ -664,7 +664,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Mantener el objetivo del núcleo: 0.66× de exposición.</t>
+          <t>Mantener el objetivo del núcleo: 0.76× de exposición.</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>{"certificadas": [], "forward": {"S01 Parabolic SAR + EMA200": {"retorno": -0.021208204502223826, "caida_max": 0.030221347464636117, "ops": 3, "dias": 8, "sharpe": null, "posicion_actual": 1.0}, "S02 Ichimoku": {"retorno": -0.013880228302163289, "caida_max": 0.03405983944279534, "ops": 2, "dias": 8, "sharpe": null, "posicion_actual": 1.0}, "S03 Bollinger + RSI (reversi\u00f3n)": {"retorno": 0.011763122737633136, "caida_max": 0.025601434163612047, "ops": 1, "dias": 8, "sharpe": null, "posicion_actual": 0.0}, "S04 Keltner ruptura": {"retorno": -0.041404541369365444, "caida_max": 0.041404541369365444, "ops": 2, "dias": 8, "sharpe": null, "posicion_actual": 0.0}, "S05 RSI(2) retroceso (largo)": {"retorno": 0.0, "caida_max": 0.0, "ops": 0, "dias": 8, "sharpe": null, "posicion_actual": 0.0}, "S06 Cruce SMA 7-25": {"retorno": 0.013110026589452373, "caida_max": 0.024438765486139102, "ops": 2, "dias": 8, "sharpe": null, "posicion_actual": 1.0}, "S07 SMA 7-25 + filtro 200 (largo)": {"retorno": 0.01827895370899535, "caida_max": 0.02443876548613899, "ops": 1, "dias": 8, "sharpe": null, "posicion_actual": 1.0}, "S08 Canal 20 por tercios": {"retorno": -0.04008285523508004, "caida_max": 0.04338030729755338, "ops": 7, "dias": 8, "sharpe": null, "posicion_actual": 0.0}, "S09 Donchian 20/10": {"retorno": -0.03748016547649924, "caida_max": 0.05407147927571376, "ops": 2, "dias": 8, "sharpe": null, "posicion_actual": 1.0}, "S10 MACD + EMA200": {"retorno": 0.0073257834870295024, "caida_max": 0.024438765486139102, "ops": 2, "dias": 8, "sharpe": null, "posicion_actual": 0.0}, "S11 Supertrend 10/3": {"retorno": -0.024343698875659014, "caida_max": 0.0411614508549194, "ops": 2, "dias": 8, "sharpe": null, "posicion_actual": 1.0}, "S12 Expansi\u00f3n de volatilidad": {"retorno": -0.01814174437269811, "caida_max": 0.024438765486139102, "ops": 3, "dias": 8, "sharpe": null, "posicion_actual": 0.0}, "S13 Retroceso a EMA20": {"retorno": 0.010589949331175408, "caida_max": 0.02443876548613899, "ops": 2, "dias": 8, "sharpe": null, "posicion_actual": 1.0}, "S14 Momentum 90 d": {"retorno": 0.02185982878057202, "caida_max": 0.02443876548613899, "ops": 1, "dias": 8, "sharpe": null, "posicion_actual": 1.0}, "S15 RSI14 + EMA200": {"retorno": 0.009306187460898618, "caida_max": 0.024438765486139213, "ops": 1, "dias": 8, "sharpe": null, "posicion_actual": 1.0}}}</t>
+          <t>{"certificadas": [], "forward": {"S01 Parabolic SAR + EMA200": {"retorno": -0.03793747623420063, "caida_max": 0.04355546257514298, "ops": 3, "dias": 9, "sharpe": null, "posicion_actual": 0.0}, "S02 Ichimoku": {"retorno": -0.021916178968034106, "caida_max": 0.04792737850644191, "ops": 3, "dias": 9, "sharpe": null, "posicion_actual": -1.0}, "S03 Bollinger + RSI (reversi\u00f3n)": {"retorno": 0.011763122737633136, "caida_max": 0.025601434163612047, "ops": 1, "dias": 9, "sharpe": null, "posicion_actual": 0.0}, "S04 Keltner ruptura": {"retorno": -0.041404541369365444, "caida_max": 0.041404541369365444, "ops": 2, "dias": 9, "sharpe": null, "posicion_actual": 0.0}, "S05 RSI(2) retroceso (largo)": {"retorno": -0.01043889482683169, "caida_max": 0.01043889482683169, "ops": 1, "dias": 9, "sharpe": null, "posicion_actual": 1.0}, "S06 Cruce SMA 7-25": {"retorno": 0.004689473154794621, "caida_max": 0.027573041067091464, "ops": 3, "dias": 9, "sharpe": null, "posicion_actual": -1.0}, "S07 SMA 7-25 + filtro 200 (largo)": {"retorno": 0.0007896043088966298, "caida_max": 0.028253739938344347, "ops": 1, "dias": 9, "sharpe": null, "posicion_actual": 0.0}, "S08 Canal 20 por tercios": {"retorno": -0.031348919640936335, "caida_max": 0.043968534368210466, "ops": 8, "dias": 9, "sharpe": null, "posicion_actual": -1.0}, "S09 Donchian 20/10": {"retorno": -0.045323798802941795, "caida_max": 0.057341114654743675, "ops": 3, "dias": 9, "sharpe": null, "posicion_actual": -1.0}, "S10 MACD + EMA200": {"retorno": 0.0073257834870295024, "caida_max": 0.024438765486139102, "ops": 2, "dias": 9, "sharpe": null, "posicion_actual": 0.0}, "S11 Supertrend 10/3": {"retorno": -0.03229438207632351, "caida_max": 0.04447571020367225, "ops": 3, "dias": 9, "sharpe": null, "posicion_actual": -1.0}, "S12 Expansi\u00f3n de volatilidad": {"retorno": -0.019432368835005986, "caida_max": 0.024438765486139102, "ops": 4, "dias": 9, "sharpe": null, "posicion_actual": 0.0}, "S13 Retroceso a EMA20": {"retorno": -0.006682808725984146, "caida_max": 0.02817103894115458, "ops": 2, "dias": 9, "sharpe": null, "posicion_actual": 0.0}, "S14 Momentum 90 d": {"retorno": -0.004697324033814176, "caida_max": 0.03696802905025898, "ops": 1, "dias": 9, "sharpe": null, "posicion_actual": 1.0}, "S15 RSI14 + EMA200": {"retorno": -0.007944628850053204, "caida_max": 0.02817103894115447, "ops": 1, "dias": 9, "sharpe": null, "posicion_actual": 0.0}}}</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>{"n_pruebas": 75, "etapas": {"descartada (E1/E2)": 54, "E3 sombra": 21}, "adoptables": [], "top_forward": [], "ultima_actualizacion": "2026-10-08 04:17:48.009895+00:00"}</t>
+          <t>{"n_pruebas": 75, "etapas": {"descartada (E1/E2)": 54, "E3 sombra": 21}, "adoptables": [], "top_forward": [], "ultima_actualizacion": "2026-10-09 04:17:55.538927+00:00"}</t>
         </is>
       </c>
     </row>
@@ -703,7 +703,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I45"/>
+  <dimension ref="A1:I51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2028,6 +2028,196 @@
         <v>-0.0040164791576372</v>
       </c>
       <c r="I45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-10-07 04:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>1002.979448024174</v>
+      </c>
+      <c r="C46" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="D46" t="n">
+        <v>84104.89999999999</v>
+      </c>
+      <c r="E46" t="n">
+        <v>0.5869854074874424</v>
+      </c>
+      <c r="F46" t="n">
+        <v>1</v>
+      </c>
+      <c r="G46" t="n">
+        <v>0.7439414588440338</v>
+      </c>
+      <c r="H46" t="n">
+        <v>0</v>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>OMITIDA_MIN_ORDEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-10-07 08:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>1002.92934515007</v>
+      </c>
+      <c r="C47" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="D47" t="n">
+        <v>84094.7</v>
+      </c>
+      <c r="E47" t="n">
+        <v>0.5869435397883561</v>
+      </c>
+      <c r="F47" t="n">
+        <v>1</v>
+      </c>
+      <c r="G47" t="n">
+        <v>0.7466854038718346</v>
+      </c>
+      <c r="H47" t="n">
+        <v>-0.0212971258958894</v>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>OMITIDA_MIN_ORDEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-10-07 12:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>1000.21264515007</v>
+      </c>
+      <c r="C48" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="D48" t="n">
+        <v>83706.60000000001</v>
+      </c>
+      <c r="E48" t="n">
+        <v>0.585821627872027</v>
+      </c>
+      <c r="F48" t="n">
+        <v>1</v>
+      </c>
+      <c r="G48" t="n">
+        <v>0.7480790091435656</v>
+      </c>
+      <c r="H48" t="n">
+        <v>0</v>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>OMITIDA_MIN_ORDEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-10-07 16:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>998.1407820199709</v>
+      </c>
+      <c r="C49" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="D49" t="n">
+        <v>83411.2</v>
+      </c>
+      <c r="E49" t="n">
+        <v>0.5849659792663573</v>
+      </c>
+      <c r="F49" t="n">
+        <v>1</v>
+      </c>
+      <c r="G49" t="n">
+        <v>0.7500171979425151</v>
+      </c>
+      <c r="H49" t="n">
+        <v>0.0040631300991464</v>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>OMITIDA_MIN_ORDEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-10-07 20:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>997.9407063201108</v>
+      </c>
+      <c r="C50" t="n">
+        <v>0.008999999999999999</v>
+      </c>
+      <c r="D50" t="n">
+        <v>83399.3</v>
+      </c>
+      <c r="E50" t="n">
+        <v>0.7521425824664488</v>
+      </c>
+      <c r="F50" t="n">
+        <v>1</v>
+      </c>
+      <c r="G50" t="n">
+        <v>0.7527861299349561</v>
+      </c>
+      <c r="H50" t="n">
+        <v>0</v>
+      </c>
+      <c r="I50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-10-08 00:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>996.8922903113749</v>
+      </c>
+      <c r="C51" t="n">
+        <v>0.008999999999999999</v>
+      </c>
+      <c r="D51" t="n">
+        <v>83281.89999999999</v>
+      </c>
+      <c r="E51" t="n">
+        <v>0.7518737051982671</v>
+      </c>
+      <c r="F51" t="n">
+        <v>1</v>
+      </c>
+      <c r="G51" t="n">
+        <v>0.7554058196201933</v>
+      </c>
+      <c r="H51" t="n">
+        <v>-0.008183991264230001</v>
+      </c>
+      <c r="I51" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2040,7 +2230,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2123,6 +2313,41 @@
       </c>
       <c r="I2" t="n">
         <v>0.5851764380923165</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-10-07 20:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="E3" t="n">
+        <v>83415.97986000001</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.08341597986</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>BANDA</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>0.5849313396443417</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.7521425824664488</v>
       </c>
     </row>
   </sheetData>
@@ -2222,33 +2447,33 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>12.79764802417412</v>
+        <v>-3.10770968862505</v>
       </c>
       <c r="F2" t="n">
-        <v>0.0127976480241741</v>
+        <v>-0.003107709688625</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>GANA (no realizado)</t>
+          <t>PIERDE (no realizado)</t>
         </is>
       </c>
       <c r="H2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I2" t="n">
-        <v>83579.11248</v>
+        <v>83542.86078666667</v>
       </c>
       <c r="J2" t="n">
-        <v>0.0347417845660282</v>
+        <v>0.0351907893223899</v>
       </c>
       <c r="K2" t="n">
-        <v>-0.0038324465347324</v>
+        <v>-0.0034001802666542</v>
       </c>
       <c r="L2" t="n">
         <v>0.875</v>
       </c>
       <c r="M2" t="n">
-        <v>7.166666666666667</v>
+        <v>8.166666666666666</v>
       </c>
     </row>
   </sheetData>
@@ -2262,7 +2487,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:N3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2359,18 +2584,18 @@
         <v>83579.11248</v>
       </c>
       <c r="G2" t="n">
-        <v>12.79764802417422</v>
+        <v>-2.757952653490232</v>
       </c>
       <c r="H2" t="n">
-        <v>0.0218743101927814</v>
+        <v>-0.0047140155539121</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>GANA (no realizado)</t>
+          <t>PIERDE (no realizado)</t>
         </is>
       </c>
       <c r="J2" t="n">
-        <v>0.4085377221458068</v>
+        <v>0.3849383998102183</v>
       </c>
       <c r="K2" t="n">
         <v>0.0347417845660282</v>
@@ -2382,6 +2607,56 @@
         <v>0.875</v>
       </c>
       <c r="N2" t="inlineStr">
+        <is>
+          <t>BANDA</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-10-07 20:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>ABIERTO</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="F3" t="n">
+        <v>83415.97986000001</v>
+      </c>
+      <c r="G3" t="n">
+        <v>-0.3497570351346408</v>
+      </c>
+      <c r="H3" t="n">
+        <v>-0.002096463026159</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>PIERDE (no realizado)</t>
+        </is>
+      </c>
+      <c r="J3" t="n">
+        <v>-0.0018186647253844</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" t="n">
+        <v>-0.0016073642031784</v>
+      </c>
+      <c r="M3" t="n">
+        <v>1</v>
+      </c>
+      <c r="N3" t="inlineStr">
         <is>
           <t>BANDA</t>
         </is>
@@ -2445,20 +2720,20 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>-0.02120820450222383</v>
+        <v>-0.03793747623420063</v>
       </c>
       <c r="C2" t="n">
-        <v>0.03022134746463612</v>
+        <v>0.04355546257514298</v>
       </c>
       <c r="D2" t="n">
         <v>3</v>
       </c>
       <c r="E2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -2468,20 +2743,20 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>-0.01388022830216329</v>
+        <v>-0.02191617896803411</v>
       </c>
       <c r="C3" t="n">
-        <v>0.03405983944279534</v>
+        <v>0.04792737850644191</v>
       </c>
       <c r="D3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E3" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="4">
@@ -2500,7 +2775,7 @@
         <v>1</v>
       </c>
       <c r="E4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="n">
@@ -2523,7 +2798,7 @@
         <v>2</v>
       </c>
       <c r="E5" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="n">
@@ -2537,20 +2812,20 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0</v>
+        <v>-0.01043889482683169</v>
       </c>
       <c r="C6" t="n">
-        <v>0</v>
+        <v>0.01043889482683169</v>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -2560,20 +2835,20 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.01311002658945237</v>
+        <v>0.004689473154794621</v>
       </c>
       <c r="C7" t="n">
-        <v>0.0244387654861391</v>
+        <v>0.02757304106709146</v>
       </c>
       <c r="D7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E7" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="8">
@@ -2583,20 +2858,20 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.01827895370899535</v>
+        <v>0.0007896043088966298</v>
       </c>
       <c r="C8" t="n">
-        <v>0.02443876548613899</v>
+        <v>0.02825373993834435</v>
       </c>
       <c r="D8" t="n">
         <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -2606,20 +2881,20 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>-0.04008285523508004</v>
+        <v>-0.03134891964093633</v>
       </c>
       <c r="C9" t="n">
-        <v>0.04338030729755338</v>
+        <v>0.04396853436821047</v>
       </c>
       <c r="D9" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E9" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="10">
@@ -2629,20 +2904,20 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>-0.03748016547649924</v>
+        <v>-0.04532379880294179</v>
       </c>
       <c r="C10" t="n">
-        <v>0.05407147927571376</v>
+        <v>0.05734111465474367</v>
       </c>
       <c r="D10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E10" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="11">
@@ -2661,7 +2936,7 @@
         <v>2</v>
       </c>
       <c r="E11" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="n">
@@ -2675,20 +2950,20 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>-0.02434369887565901</v>
+        <v>-0.03229438207632351</v>
       </c>
       <c r="C12" t="n">
-        <v>0.0411614508549194</v>
+        <v>0.04447571020367225</v>
       </c>
       <c r="D12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E12" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="13">
@@ -2698,16 +2973,16 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>-0.01814174437269811</v>
+        <v>-0.01943236883500599</v>
       </c>
       <c r="C13" t="n">
         <v>0.0244387654861391</v>
       </c>
       <c r="D13" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E13" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="n">
@@ -2721,20 +2996,20 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.01058994933117541</v>
+        <v>-0.006682808725984146</v>
       </c>
       <c r="C14" t="n">
-        <v>0.02443876548613899</v>
+        <v>0.02817103894115458</v>
       </c>
       <c r="D14" t="n">
         <v>2</v>
       </c>
       <c r="E14" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -2744,16 +3019,16 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.02185982878057202</v>
+        <v>-0.004697324033814176</v>
       </c>
       <c r="C15" t="n">
-        <v>0.02443876548613899</v>
+        <v>0.03696802905025898</v>
       </c>
       <c r="D15" t="n">
         <v>1</v>
       </c>
       <c r="E15" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="n">
@@ -2767,20 +3042,20 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.009306187460898618</v>
+        <v>-0.007944628850053204</v>
       </c>
       <c r="C16" t="n">
-        <v>0.02443876548613921</v>
+        <v>0.02817103894115447</v>
       </c>
       <c r="D16" t="n">
         <v>1</v>
       </c>
       <c r="E16" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
paper: actualización diaria 2026-10-10
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AtSxiX9NxnepDF7aXKR3KZ
</commit_message>
<xml_diff>
--- a/millonary/paper_state/semanal/diario.xlsx
+++ b/millonary/paper_state/semanal/diario.xlsx
@@ -442,7 +442,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-09 04:17:55.538927+00:00</t>
+          <t>2026-10-10 04:18:01.351761+00:00</t>
         </is>
       </c>
     </row>
@@ -473,7 +473,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>996.8922903113749</v>
+        <v>981.5278954506448</v>
       </c>
     </row>
     <row r="6">
@@ -483,7 +483,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>-0.002699300837112895</v>
+        <v>-0.01806999021423183</v>
       </c>
     </row>
     <row r="7">
@@ -493,7 +493,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>-0.01568942775918525</v>
+        <v>-0.02524173958615039</v>
       </c>
     </row>
     <row r="8">
@@ -503,7 +503,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.02229207276637357</v>
+        <v>0.03947605203802207</v>
       </c>
     </row>
     <row r="9">
@@ -513,7 +513,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.02229207276637357</v>
+        <v>0.03736079262555858</v>
       </c>
     </row>
     <row r="10">
@@ -523,7 +523,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="11">
@@ -533,7 +533,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>50</v>
+        <v>56</v>
       </c>
     </row>
     <row r="12">
@@ -543,7 +543,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.7518737051982671</v>
+        <v>0.2497463405127708</v>
       </c>
     </row>
     <row r="13">
@@ -563,7 +563,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15">
@@ -573,7 +573,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="16">
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.37594287354</v>
+        <v>0.6205926338</v>
       </c>
     </row>
     <row r="17">
@@ -593,7 +593,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0.08341597986</v>
+        <v>0.32806574012</v>
       </c>
     </row>
     <row r="18">
@@ -640,7 +640,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>{"dias": 9, "estado": "insuficiente"}</t>
+          <t>{"dias": 10, "sharpe_observado": -4.355659519318118, "error_estandar": 19.56360906709532, "posterior_media": 0.396895660400446, "posterior_sd": 0.4998367815044741, "prob_sharpe_mayor_0": 0.7864169918071333, "ic90": [-0.4253358451744139, 1.2191271659753058], "prior": {"media": 0.4, "sd": 0.5}}</t>
         </is>
       </c>
     </row>
@@ -664,7 +664,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Mantener el objetivo del núcleo: 0.76× de exposición.</t>
+          <t>Mantener el objetivo del núcleo: 0.28× de exposición.</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>{"certificadas": [], "forward": {"S01 Parabolic SAR + EMA200": {"retorno": -0.03793747623420063, "caida_max": 0.04355546257514298, "ops": 3, "dias": 9, "sharpe": null, "posicion_actual": 0.0}, "S02 Ichimoku": {"retorno": -0.021916178968034106, "caida_max": 0.04792737850644191, "ops": 3, "dias": 9, "sharpe": null, "posicion_actual": -1.0}, "S03 Bollinger + RSI (reversi\u00f3n)": {"retorno": 0.011763122737633136, "caida_max": 0.025601434163612047, "ops": 1, "dias": 9, "sharpe": null, "posicion_actual": 0.0}, "S04 Keltner ruptura": {"retorno": -0.041404541369365444, "caida_max": 0.041404541369365444, "ops": 2, "dias": 9, "sharpe": null, "posicion_actual": 0.0}, "S05 RSI(2) retroceso (largo)": {"retorno": -0.01043889482683169, "caida_max": 0.01043889482683169, "ops": 1, "dias": 9, "sharpe": null, "posicion_actual": 1.0}, "S06 Cruce SMA 7-25": {"retorno": 0.004689473154794621, "caida_max": 0.027573041067091464, "ops": 3, "dias": 9, "sharpe": null, "posicion_actual": -1.0}, "S07 SMA 7-25 + filtro 200 (largo)": {"retorno": 0.0007896043088966298, "caida_max": 0.028253739938344347, "ops": 1, "dias": 9, "sharpe": null, "posicion_actual": 0.0}, "S08 Canal 20 por tercios": {"retorno": -0.031348919640936335, "caida_max": 0.043968534368210466, "ops": 8, "dias": 9, "sharpe": null, "posicion_actual": -1.0}, "S09 Donchian 20/10": {"retorno": -0.045323798802941795, "caida_max": 0.057341114654743675, "ops": 3, "dias": 9, "sharpe": null, "posicion_actual": -1.0}, "S10 MACD + EMA200": {"retorno": 0.0073257834870295024, "caida_max": 0.024438765486139102, "ops": 2, "dias": 9, "sharpe": null, "posicion_actual": 0.0}, "S11 Supertrend 10/3": {"retorno": -0.03229438207632351, "caida_max": 0.04447571020367225, "ops": 3, "dias": 9, "sharpe": null, "posicion_actual": -1.0}, "S12 Expansi\u00f3n de volatilidad": {"retorno": -0.019432368835005986, "caida_max": 0.024438765486139102, "ops": 4, "dias": 9, "sharpe": null, "posicion_actual": 0.0}, "S13 Retroceso a EMA20": {"retorno": -0.006682808725984146, "caida_max": 0.02817103894115458, "ops": 2, "dias": 9, "sharpe": null, "posicion_actual": 0.0}, "S14 Momentum 90 d": {"retorno": -0.004697324033814176, "caida_max": 0.03696802905025898, "ops": 1, "dias": 9, "sharpe": null, "posicion_actual": 1.0}, "S15 RSI14 + EMA200": {"retorno": -0.007944628850053204, "caida_max": 0.02817103894115447, "ops": 1, "dias": 9, "sharpe": null, "posicion_actual": 0.0}}}</t>
+          <t>{"certificadas": [], "forward": {"S01 Parabolic SAR + EMA200": {"retorno": -0.048095263465906535, "caida_max": 0.053653933173561374, "ops": 4, "dias": 10, "sharpe": -14.726107860828897, "posicion_actual": 0.0}, "S02 Ichimoku": {"retorno": -0.0035661661296337854, "caida_max": 0.04792737850644191, "ops": 3, "dias": 10, "sharpe": -0.8095873373892396, "posicion_actual": -1.0}, "S03 Bollinger + RSI (reversi\u00f3n)": {"retorno": 0.020036096411532478, "caida_max": 0.025601434163612047, "ops": 2, "dias": 10, "sharpe": 3.512173247518957, "posicion_actual": 1.0}, "S04 Keltner ruptura": {"retorno": -0.030677093522502363, "caida_max": 0.044762968367285105, "ops": 3, "dias": 10, "sharpe": -5.683574990345989, "posicion_actual": -1.0}, "S05 RSI(2) retroceso (largo)": {"retorno": -0.029140530487063, "caida_max": 0.03768262617940443, "ops": 1, "dias": 10, "sharpe": -8.625102163836981, "posicion_actual": 1.0}, "S06 Cruce SMA 7-25": {"retorno": 0.02353863959080038, "caida_max": 0.027573041067091464, "ops": 3, "dias": 10, "sharpe": 4.427907875174454, "posicion_actual": -1.0}, "S07 SMA 7-25 + filtro 200 (largo)": {"retorno": 0.0007896043088966298, "caida_max": 0.028253739938344347, "ops": 1, "dias": 10, "sharpe": 0.23495927627192095, "posicion_actual": 0.0}, "S08 Canal 20 por tercios": {"retorno": -0.013175876208150528, "caida_max": 0.043968534368210466, "ops": 8, "dias": 10, "sharpe": -2.361791904094518, "posicion_actual": -1.0}, "S09 Donchian 20/10": {"retorno": -0.02741294068242006, "caida_max": 0.057341114654743675, "ops": 3, "dias": 10, "sharpe": -3.2273947181336875, "posicion_actual": -1.0}, "S10 MACD + EMA200": {"retorno": -0.0033099088187271697, "caida_max": 0.031043992676942023, "ops": 3, "dias": 10, "sharpe": -0.6647363374726754, "posicion_actual": 0.0}, "S11 Supertrend 10/3": {"retorno": -0.014139076640480752, "caida_max": 0.04447571020367225, "ops": 3, "dias": 10, "sharpe": -1.9447712785819689, "posicion_actual": -1.0}, "S12 Expansi\u00f3n de volatilidad": {"retorno": -0.02882819959249816, "caida_max": 0.0318579706938229, "ops": 5, "dias": 10, "sharpe": -10.900692302667261, "posicion_actual": -1.0}, "S13 Retroceso a EMA20": {"retorno": -0.006682808725984146, "caida_max": 0.02817103894115458, "ops": 2, "dias": 10, "sharpe": -1.1915110981942436, "posicion_actual": 0.0}, "S14 Momentum 90 d": {"retorno": -0.02350746917822688, "caida_max": 0.06348138346903642, "ops": 1, "dias": 10, "sharpe": -3.142693006790305, "posicion_actual": 1.0}, "S15 RSI14 + EMA200": {"retorno": -0.01745053550364284, "caida_max": 0.037758374441150155, "ops": 2, "dias": 10, "sharpe": -3.2783360218243485, "posicion_actual": -1.0}}}</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>{"n_pruebas": 75, "etapas": {"descartada (E1/E2)": 54, "E3 sombra": 21}, "adoptables": [], "top_forward": [], "ultima_actualizacion": "2026-10-09 04:17:55.538927+00:00"}</t>
+          <t>{"n_pruebas": 75, "etapas": {"descartada (E1/E2)": 54, "E3 sombra": 21}, "adoptables": [], "top_forward": [["S01 Parabolic SAR + EMA200|O3 tama\u00f1o por volatilidad", {"dias": 10, "delta_sharpe": 0.0, "caida_base": 0.04806307582208469, "caida_var": 0.03588632361481847, "ret_base": -0.048095263465906646, "ret_var": -0.035909097673150425, "p_boot": null}], ["S02 Ichimoku|O2 solo largos", {"dias": 10, "delta_sharpe": 0.0, "caida_base": 0.021916178968034217, "caida_var": 0.03073474802422349, "ret_base": -0.0035661661296341185, "ret_var": -0.03073474802422349, "p_boot": null}], ["S02 Ichimoku|O3 tama\u00f1o por volatilidad", {"dias": 10, "delta_sharpe": 0.0, "caida_base": 0.021916178968034217, "caida_var": 0.0165006851857864, "ret_base": -0.0035661661296341185, "ret_var": -0.002388520497693225, "p_boot": null}], ["S03 Bollinger + RSI (reversi\u00f3n)|O2 solo largos", {"dias": 10, "delta_sharpe": 0.0, "caida_base": 0.02314550224080769, "caida_var": 0.0, "ret_base": 0.020036096411532256, "ret_var": 0.00817678910011499, "p_boot": null}], ["S03 Bollinger + RSI (reversi\u00f3n)|O4 stop 3\u00d7ATR", {"dias": 10, "delta_sharpe": 0.0, "caida_base": 0.02314550224080769, "caida_var": 0.02382930038923925, "ret_base": 0.020036096411532256, "ret_var": 0.00527059403948793, "p_boot": null}]], "ultima_actualizacion": "2026-10-10 04:18:01.351761+00:00"}</t>
         </is>
       </c>
     </row>
@@ -703,7 +703,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I51"/>
+  <dimension ref="A1:I57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2218,6 +2218,180 @@
         <v>-0.008183991264230001</v>
       </c>
       <c r="I51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-10-08 04:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>991.6951026348352</v>
+      </c>
+      <c r="C52" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="D52" t="n">
+        <v>82717.3</v>
+      </c>
+      <c r="E52" t="n">
+        <v>0.5838700810981103</v>
+      </c>
+      <c r="F52" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="G52" t="n">
+        <v>0.6609502348652737</v>
+      </c>
+      <c r="H52" t="n">
+        <v>0</v>
+      </c>
+      <c r="I52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-10-08 08:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>993.3183984577402</v>
+      </c>
+      <c r="C53" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="D53" t="n">
+        <v>82948.3</v>
+      </c>
+      <c r="E53" t="n">
+        <v>0.5845437886799625</v>
+      </c>
+      <c r="F53" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="G53" t="n">
+        <v>0.6630960102340053</v>
+      </c>
+      <c r="H53" t="n">
+        <v>-0.0062958229050568</v>
+      </c>
+      <c r="I53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-10-08 12:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>989.9303984577402</v>
+      </c>
+      <c r="C54" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="D54" t="n">
+        <v>82464.3</v>
+      </c>
+      <c r="E54" t="n">
+        <v>0.5831219052362929</v>
+      </c>
+      <c r="F54" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="G54" t="n">
+        <v>0.6636885873201623</v>
+      </c>
+      <c r="H54" t="n">
+        <v>0</v>
+      </c>
+      <c r="I54" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-10-08 16:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>979.371130898004</v>
+      </c>
+      <c r="C55" t="n">
+        <v>0.003</v>
+      </c>
+      <c r="D55" t="n">
+        <v>80990.7</v>
+      </c>
+      <c r="E55" t="n">
+        <v>0.2480899143690444</v>
+      </c>
+      <c r="F55" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="G55" t="n">
+        <v>0.2787254532064649</v>
+      </c>
+      <c r="H55" t="n">
+        <v>0.0173259960160185</v>
+      </c>
+      <c r="I55" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-10-08 20:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>981.598030898004</v>
+      </c>
+      <c r="C56" t="n">
+        <v>0.003</v>
+      </c>
+      <c r="D56" t="n">
+        <v>81733</v>
+      </c>
+      <c r="E56" t="n">
+        <v>0.2497957333672343</v>
+      </c>
+      <c r="F56" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="G56" t="n">
+        <v>0.2781364840185184</v>
+      </c>
+      <c r="H56" t="n">
+        <v>0</v>
+      </c>
+      <c r="I56" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-10-09 00:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>981.5278954506448</v>
+      </c>
+      <c r="C57" t="n">
+        <v>0.003</v>
+      </c>
+      <c r="D57" t="n">
+        <v>81711</v>
+      </c>
+      <c r="E57" t="n">
+        <v>0.2497463405127708</v>
+      </c>
+      <c r="F57" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="G57" t="n">
+        <v>0.2791641491221762</v>
+      </c>
+      <c r="H57" t="n">
+        <v>0.0041354473593871</v>
+      </c>
+      <c r="I57" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2230,7 +2404,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2348,6 +2522,76 @@
       </c>
       <c r="I3" t="n">
         <v>0.7521425824664488</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-10-08 04:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>-0.002</v>
+      </c>
+      <c r="E4" t="n">
+        <v>82700.75654</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.08270075654</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>SEÑAL</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>0.7506024659260206</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.5838700810981103</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-10-08 16:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>-0.004</v>
+      </c>
+      <c r="E5" t="n">
+        <v>80974.50186</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.16194900372</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>SEÑAL</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>0.5787424778448076</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.2480899143690444</v>
       </c>
     </row>
   </sheetData>
@@ -2447,10 +2691,10 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>-3.10770968862505</v>
+        <v>-18.47210454935532</v>
       </c>
       <c r="F2" t="n">
-        <v>-0.003107709688625</v>
+        <v>-0.0184721045493553</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -2467,13 +2711,13 @@
         <v>0.0351907893223899</v>
       </c>
       <c r="K2" t="n">
-        <v>-0.0034001802666542</v>
+        <v>-0.0305491188910064</v>
       </c>
       <c r="L2" t="n">
         <v>0.875</v>
       </c>
       <c r="M2" t="n">
-        <v>8.166666666666666</v>
+        <v>9.166666666666666</v>
       </c>
     </row>
   </sheetData>
@@ -2584,10 +2828,10 @@
         <v>83579.11248</v>
       </c>
       <c r="G2" t="n">
-        <v>-2.757952653490232</v>
+        <v>-14.97463907128256</v>
       </c>
       <c r="H2" t="n">
-        <v>-0.0047140155539121</v>
+        <v>-0.0255953202847454</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -2595,13 +2839,13 @@
         </is>
       </c>
       <c r="J2" t="n">
-        <v>0.3849383998102183</v>
+        <v>0.3941955773426058</v>
       </c>
       <c r="K2" t="n">
         <v>0.0347417845660282</v>
       </c>
       <c r="L2" t="n">
-        <v>-0.0038324465347324</v>
+        <v>-0.0309696095495078</v>
       </c>
       <c r="M2" t="n">
         <v>0.875</v>
@@ -2634,10 +2878,10 @@
         <v>83415.97986000001</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.3497570351346408</v>
+        <v>-3.497465478072592</v>
       </c>
       <c r="H3" t="n">
-        <v>-0.002096463026159</v>
+        <v>-0.0209640016453832</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
@@ -2645,13 +2889,13 @@
         </is>
       </c>
       <c r="J3" t="n">
-        <v>-0.0018186647253844</v>
+        <v>0.0040897782125769</v>
       </c>
       <c r="K3" t="n">
         <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>-0.0016073642031784</v>
+        <v>-0.0290745234194987</v>
       </c>
       <c r="M3" t="n">
         <v>1</v>
@@ -2720,18 +2964,20 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>-0.03793747623420063</v>
+        <v>-0.04809526346590653</v>
       </c>
       <c r="C2" t="n">
-        <v>0.04355546257514298</v>
+        <v>0.05365393317356137</v>
       </c>
       <c r="D2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E2" t="n">
-        <v>9</v>
-      </c>
-      <c r="F2" t="inlineStr"/>
+        <v>10</v>
+      </c>
+      <c r="F2" t="n">
+        <v>-14.7261078608289</v>
+      </c>
       <c r="G2" t="n">
         <v>0</v>
       </c>
@@ -2743,7 +2989,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>-0.02191617896803411</v>
+        <v>-0.003566166129633785</v>
       </c>
       <c r="C3" t="n">
         <v>0.04792737850644191</v>
@@ -2752,9 +2998,11 @@
         <v>3</v>
       </c>
       <c r="E3" t="n">
-        <v>9</v>
-      </c>
-      <c r="F3" t="inlineStr"/>
+        <v>10</v>
+      </c>
+      <c r="F3" t="n">
+        <v>-0.8095873373892396</v>
+      </c>
       <c r="G3" t="n">
         <v>-1</v>
       </c>
@@ -2766,20 +3014,22 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.01176312273763314</v>
+        <v>0.02003609641153248</v>
       </c>
       <c r="C4" t="n">
         <v>0.02560143416361205</v>
       </c>
       <c r="D4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E4" t="n">
+        <v>10</v>
+      </c>
+      <c r="F4" t="n">
+        <v>3.512173247518957</v>
+      </c>
+      <c r="G4" t="n">
         <v>1</v>
-      </c>
-      <c r="E4" t="n">
-        <v>9</v>
-      </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -2789,20 +3039,22 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>-0.04140454136936544</v>
+        <v>-0.03067709352250236</v>
       </c>
       <c r="C5" t="n">
-        <v>0.04140454136936544</v>
+        <v>0.04476296836728511</v>
       </c>
       <c r="D5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E5" t="n">
-        <v>9</v>
-      </c>
-      <c r="F5" t="inlineStr"/>
+        <v>10</v>
+      </c>
+      <c r="F5" t="n">
+        <v>-5.683574990345989</v>
+      </c>
       <c r="G5" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="6">
@@ -2812,18 +3064,20 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>-0.01043889482683169</v>
+        <v>-0.029140530487063</v>
       </c>
       <c r="C6" t="n">
-        <v>0.01043889482683169</v>
+        <v>0.03768262617940443</v>
       </c>
       <c r="D6" t="n">
         <v>1</v>
       </c>
       <c r="E6" t="n">
-        <v>9</v>
-      </c>
-      <c r="F6" t="inlineStr"/>
+        <v>10</v>
+      </c>
+      <c r="F6" t="n">
+        <v>-8.625102163836981</v>
+      </c>
       <c r="G6" t="n">
         <v>1</v>
       </c>
@@ -2835,7 +3089,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.004689473154794621</v>
+        <v>0.02353863959080038</v>
       </c>
       <c r="C7" t="n">
         <v>0.02757304106709146</v>
@@ -2844,9 +3098,11 @@
         <v>3</v>
       </c>
       <c r="E7" t="n">
-        <v>9</v>
-      </c>
-      <c r="F7" t="inlineStr"/>
+        <v>10</v>
+      </c>
+      <c r="F7" t="n">
+        <v>4.427907875174454</v>
+      </c>
       <c r="G7" t="n">
         <v>-1</v>
       </c>
@@ -2867,9 +3123,11 @@
         <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>9</v>
-      </c>
-      <c r="F8" t="inlineStr"/>
+        <v>10</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.234959276271921</v>
+      </c>
       <c r="G8" t="n">
         <v>0</v>
       </c>
@@ -2881,7 +3139,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>-0.03134891964093633</v>
+        <v>-0.01317587620815053</v>
       </c>
       <c r="C9" t="n">
         <v>0.04396853436821047</v>
@@ -2890,9 +3148,11 @@
         <v>8</v>
       </c>
       <c r="E9" t="n">
-        <v>9</v>
-      </c>
-      <c r="F9" t="inlineStr"/>
+        <v>10</v>
+      </c>
+      <c r="F9" t="n">
+        <v>-2.361791904094518</v>
+      </c>
       <c r="G9" t="n">
         <v>-1</v>
       </c>
@@ -2904,7 +3164,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>-0.04532379880294179</v>
+        <v>-0.02741294068242006</v>
       </c>
       <c r="C10" t="n">
         <v>0.05734111465474367</v>
@@ -2913,9 +3173,11 @@
         <v>3</v>
       </c>
       <c r="E10" t="n">
-        <v>9</v>
-      </c>
-      <c r="F10" t="inlineStr"/>
+        <v>10</v>
+      </c>
+      <c r="F10" t="n">
+        <v>-3.227394718133688</v>
+      </c>
       <c r="G10" t="n">
         <v>-1</v>
       </c>
@@ -2927,18 +3189,20 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.007325783487029502</v>
+        <v>-0.00330990881872717</v>
       </c>
       <c r="C11" t="n">
-        <v>0.0244387654861391</v>
+        <v>0.03104399267694202</v>
       </c>
       <c r="D11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E11" t="n">
-        <v>9</v>
-      </c>
-      <c r="F11" t="inlineStr"/>
+        <v>10</v>
+      </c>
+      <c r="F11" t="n">
+        <v>-0.6647363374726754</v>
+      </c>
       <c r="G11" t="n">
         <v>0</v>
       </c>
@@ -2950,7 +3214,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>-0.03229438207632351</v>
+        <v>-0.01413907664048075</v>
       </c>
       <c r="C12" t="n">
         <v>0.04447571020367225</v>
@@ -2959,9 +3223,11 @@
         <v>3</v>
       </c>
       <c r="E12" t="n">
-        <v>9</v>
-      </c>
-      <c r="F12" t="inlineStr"/>
+        <v>10</v>
+      </c>
+      <c r="F12" t="n">
+        <v>-1.944771278581969</v>
+      </c>
       <c r="G12" t="n">
         <v>-1</v>
       </c>
@@ -2973,20 +3239,22 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>-0.01943236883500599</v>
+        <v>-0.02882819959249816</v>
       </c>
       <c r="C13" t="n">
-        <v>0.0244387654861391</v>
+        <v>0.0318579706938229</v>
       </c>
       <c r="D13" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E13" t="n">
-        <v>9</v>
-      </c>
-      <c r="F13" t="inlineStr"/>
+        <v>10</v>
+      </c>
+      <c r="F13" t="n">
+        <v>-10.90069230266726</v>
+      </c>
       <c r="G13" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="14">
@@ -3005,9 +3273,11 @@
         <v>2</v>
       </c>
       <c r="E14" t="n">
-        <v>9</v>
-      </c>
-      <c r="F14" t="inlineStr"/>
+        <v>10</v>
+      </c>
+      <c r="F14" t="n">
+        <v>-1.191511098194244</v>
+      </c>
       <c r="G14" t="n">
         <v>0</v>
       </c>
@@ -3019,18 +3289,20 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>-0.004697324033814176</v>
+        <v>-0.02350746917822688</v>
       </c>
       <c r="C15" t="n">
-        <v>0.03696802905025898</v>
+        <v>0.06348138346903642</v>
       </c>
       <c r="D15" t="n">
         <v>1</v>
       </c>
       <c r="E15" t="n">
-        <v>9</v>
-      </c>
-      <c r="F15" t="inlineStr"/>
+        <v>10</v>
+      </c>
+      <c r="F15" t="n">
+        <v>-3.142693006790305</v>
+      </c>
       <c r="G15" t="n">
         <v>1</v>
       </c>
@@ -3042,20 +3314,22 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>-0.007944628850053204</v>
+        <v>-0.01745053550364284</v>
       </c>
       <c r="C16" t="n">
-        <v>0.02817103894115447</v>
+        <v>0.03775837444115016</v>
       </c>
       <c r="D16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E16" t="n">
-        <v>9</v>
-      </c>
-      <c r="F16" t="inlineStr"/>
+        <v>10</v>
+      </c>
+      <c r="F16" t="n">
+        <v>-3.278336021824348</v>
+      </c>
       <c r="G16" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
   </sheetData>
@@ -3069,22 +3343,180 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>info</t>
+          <t>candidata</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>dias</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>delta_sharpe</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>caida_base</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>caida_var</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>ret_base</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>ret_var</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>p_boot</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>sin datos hacia delante</t>
-        </is>
-      </c>
+          <t>S01 Parabolic SAR + EMA200|O3 tamaño por volatilidad</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>10</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.04806307582208469</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.03588632361481847</v>
+      </c>
+      <c r="F2" t="n">
+        <v>-0.04809526346590665</v>
+      </c>
+      <c r="G2" t="n">
+        <v>-0.03590909767315043</v>
+      </c>
+      <c r="H2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>S02 Ichimoku|O2 solo largos</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>10</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.02191617896803422</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.03073474802422349</v>
+      </c>
+      <c r="F3" t="n">
+        <v>-0.003566166129634118</v>
+      </c>
+      <c r="G3" t="n">
+        <v>-0.03073474802422349</v>
+      </c>
+      <c r="H3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>S02 Ichimoku|O3 tamaño por volatilidad</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>10</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.02191617896803422</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.0165006851857864</v>
+      </c>
+      <c r="F4" t="n">
+        <v>-0.003566166129634118</v>
+      </c>
+      <c r="G4" t="n">
+        <v>-0.002388520497693225</v>
+      </c>
+      <c r="H4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>S03 Bollinger + RSI (reversión)|O2 solo largos</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>10</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.02314550224080769</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.02003609641153226</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.008176789100114989</v>
+      </c>
+      <c r="H5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>S03 Bollinger + RSI (reversión)|O4 stop 3×ATR</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>10</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.02314550224080769</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.02382930038923925</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.02003609641153226</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.00527059403948793</v>
+      </c>
+      <c r="H6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
paper: actualización diaria 2026-10-11
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AtSxiX9NxnepDF7aXKR3KZ
</commit_message>
<xml_diff>
--- a/millonary/paper_state/semanal/diario.xlsx
+++ b/millonary/paper_state/semanal/diario.xlsx
@@ -442,7 +442,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-10 04:18:01.351761+00:00</t>
+          <t>2026-10-11 04:18:23.580833+00:00</t>
         </is>
       </c>
     </row>
@@ -473,7 +473,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>981.5278954506448</v>
+        <v>984.1010267234344</v>
       </c>
     </row>
     <row r="6">
@@ -483,7 +483,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>-0.01806999021423183</v>
+        <v>-0.01549580477581358</v>
       </c>
     </row>
     <row r="7">
@@ -493,7 +493,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>-0.02524173958615039</v>
+        <v>-0.02364137861763305</v>
       </c>
     </row>
     <row r="8">
@@ -513,7 +513,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.03736079262555858</v>
+        <v>0.03483717912421092</v>
       </c>
     </row>
     <row r="10">
@@ -523,7 +523,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11">
@@ -533,7 +533,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>56</v>
+        <v>62</v>
       </c>
     </row>
     <row r="12">
@@ -543,7 +543,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.2497463405127708</v>
+        <v>0.2517378737270863</v>
       </c>
     </row>
     <row r="13">
@@ -640,7 +640,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>{"dias": 10, "sharpe_observado": -4.355659519318118, "error_estandar": 19.56360906709532, "posterior_media": 0.396895660400446, "posterior_sd": 0.4998367815044741, "prob_sharpe_mayor_0": 0.7864169918071333, "ic90": [-0.4253358451744139, 1.2191271659753058], "prior": {"media": 0.4, "sd": 0.5}}</t>
+          <t>{"dias": 11, "sharpe_observado": -3.5187721302916484, "error_estandar": 15.446890561320082, "posterior_media": 0.39589840206218796, "posterior_sd": 0.49973826803385435, "prob_sharpe_mayor_0": 0.7858813173889656, "ic90": [-0.42617104885350243, 1.2179678529778784], "prior": {"media": 0.4, "sd": 0.5}}</t>
         </is>
       </c>
     </row>
@@ -652,7 +652,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>AVISO</t>
         </is>
       </c>
     </row>
@@ -664,7 +664,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Mantener el objetivo del núcleo: 0.28× de exposición.</t>
+          <t>Mantener el objetivo del núcleo: 0.38× de exposición.</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>{"certificadas": [], "forward": {"S01 Parabolic SAR + EMA200": {"retorno": -0.048095263465906535, "caida_max": 0.053653933173561374, "ops": 4, "dias": 10, "sharpe": -14.726107860828897, "posicion_actual": 0.0}, "S02 Ichimoku": {"retorno": -0.0035661661296337854, "caida_max": 0.04792737850644191, "ops": 3, "dias": 10, "sharpe": -0.8095873373892396, "posicion_actual": -1.0}, "S03 Bollinger + RSI (reversi\u00f3n)": {"retorno": 0.020036096411532478, "caida_max": 0.025601434163612047, "ops": 2, "dias": 10, "sharpe": 3.512173247518957, "posicion_actual": 1.0}, "S04 Keltner ruptura": {"retorno": -0.030677093522502363, "caida_max": 0.044762968367285105, "ops": 3, "dias": 10, "sharpe": -5.683574990345989, "posicion_actual": -1.0}, "S05 RSI(2) retroceso (largo)": {"retorno": -0.029140530487063, "caida_max": 0.03768262617940443, "ops": 1, "dias": 10, "sharpe": -8.625102163836981, "posicion_actual": 1.0}, "S06 Cruce SMA 7-25": {"retorno": 0.02353863959080038, "caida_max": 0.027573041067091464, "ops": 3, "dias": 10, "sharpe": 4.427907875174454, "posicion_actual": -1.0}, "S07 SMA 7-25 + filtro 200 (largo)": {"retorno": 0.0007896043088966298, "caida_max": 0.028253739938344347, "ops": 1, "dias": 10, "sharpe": 0.23495927627192095, "posicion_actual": 0.0}, "S08 Canal 20 por tercios": {"retorno": -0.013175876208150528, "caida_max": 0.043968534368210466, "ops": 8, "dias": 10, "sharpe": -2.361791904094518, "posicion_actual": -1.0}, "S09 Donchian 20/10": {"retorno": -0.02741294068242006, "caida_max": 0.057341114654743675, "ops": 3, "dias": 10, "sharpe": -3.2273947181336875, "posicion_actual": -1.0}, "S10 MACD + EMA200": {"retorno": -0.0033099088187271697, "caida_max": 0.031043992676942023, "ops": 3, "dias": 10, "sharpe": -0.6647363374726754, "posicion_actual": 0.0}, "S11 Supertrend 10/3": {"retorno": -0.014139076640480752, "caida_max": 0.04447571020367225, "ops": 3, "dias": 10, "sharpe": -1.9447712785819689, "posicion_actual": -1.0}, "S12 Expansi\u00f3n de volatilidad": {"retorno": -0.02882819959249816, "caida_max": 0.0318579706938229, "ops": 5, "dias": 10, "sharpe": -10.900692302667261, "posicion_actual": -1.0}, "S13 Retroceso a EMA20": {"retorno": -0.006682808725984146, "caida_max": 0.02817103894115458, "ops": 2, "dias": 10, "sharpe": -1.1915110981942436, "posicion_actual": 0.0}, "S14 Momentum 90 d": {"retorno": -0.02350746917822688, "caida_max": 0.06348138346903642, "ops": 1, "dias": 10, "sharpe": -3.142693006790305, "posicion_actual": 1.0}, "S15 RSI14 + EMA200": {"retorno": -0.01745053550364284, "caida_max": 0.037758374441150155, "ops": 2, "dias": 10, "sharpe": -3.2783360218243485, "posicion_actual": -1.0}}}</t>
+          <t>{"certificadas": [], "forward": {"S01 Parabolic SAR + EMA200": {"retorno": -0.055933527578663655, "caida_max": 0.06450512282574605, "ops": 5, "dias": 11, "sharpe": -16.25893627154939, "posicion_actual": 1.0}, "S02 Ichimoku": {"retorno": -0.014111223949835328, "caida_max": 0.04792737850644191, "ops": 3, "dias": 11, "sharpe": -3.010412212517539, "posicion_actual": -1.0}, "S03 Bollinger + RSI (reversi\u00f3n)": {"retorno": 0.03074363393482571, "caida_max": 0.025601434163612047, "ops": 2, "dias": 11, "sharpe": 4.953362339748169, "posicion_actual": 1.0}, "S04 Keltner ruptura": {"retorno": -0.040935241878974904, "caida_max": 0.04809548795047969, "ops": 3, "dias": 11, "sharpe": -7.138471252338212, "posicion_actual": -1.0}, "S05 RSI(2) retroceso (largo)": {"retorno": -0.02181633521027726, "caida_max": 0.03768262617940443, "ops": 1, "dias": 11, "sharpe": -5.464156619515538, "posicion_actual": 0.0}, "S06 Cruce SMA 7-25": {"retorno": 0.012706737091291664, "caida_max": 0.027573041067091464, "ops": 3, "dias": 11, "sharpe": 2.183788367764555, "posicion_actual": -1.0}, "S07 SMA 7-25 + filtro 200 (largo)": {"retorno": 0.0007896043088966298, "caida_max": 0.028253739938344347, "ops": 1, "dias": 11, "sharpe": 0.2251517559894329, "posicion_actual": 0.0}, "S08 Canal 20 por tercios": {"retorno": -0.028577535636180262, "caida_max": 0.043968534368210466, "ops": 9, "dias": 11, "sharpe": -4.601283393613085, "posicion_actual": 0.0}, "S09 Donchian 20/10": {"retorno": -0.03770563290850304, "caida_max": 0.057341114654743675, "ops": 3, "dias": 11, "sharpe": -4.267600760326958, "posicion_actual": -1.0}, "S10 MACD + EMA200": {"retorno": -0.007200591349226015, "caida_max": 0.03797186285349852, "ops": 4, "dias": 11, "sharpe": -1.4570621008123732, "posicion_actual": 1.0}, "S11 Supertrend 10/3": {"retorno": -0.02457224348621423, "caida_max": 0.04447571020367225, "ops": 3, "dias": 11, "sharpe": -3.250997968322616, "posicion_actual": -1.0}, "S12 Expansi\u00f3n de volatilidad": {"retorno": -0.03910591441965128, "caida_max": 0.048983194737682534, "ops": 5, "dias": 11, "sharpe": -12.85118271162761, "posicion_actual": -1.0}, "S13 Retroceso a EMA20": {"retorno": -0.006682808725984146, "caida_max": 0.02817103894115458, "ops": 2, "dias": 11, "sharpe": -1.1415602932162299, "posicion_actual": 0.0}, "S14 Momentum 90 d": {"retorno": -0.013257017795405335, "caida_max": 0.06348138346903642, "ops": 1, "dias": 11, "sharpe": -1.564867524079307, "posicion_actual": 1.0}, "S15 RSI14 + EMA200": {"retorno": -0.027848657849687264, "caida_max": 0.054779227707723366, "ops": 2, "dias": 11, "sharpe": -4.89008477566683, "posicion_actual": -1.0}}}</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>{"n_pruebas": 75, "etapas": {"descartada (E1/E2)": 54, "E3 sombra": 21}, "adoptables": [], "top_forward": [["S01 Parabolic SAR + EMA200|O3 tama\u00f1o por volatilidad", {"dias": 10, "delta_sharpe": 0.0, "caida_base": 0.04806307582208469, "caida_var": 0.03588632361481847, "ret_base": -0.048095263465906646, "ret_var": -0.035909097673150425, "p_boot": null}], ["S02 Ichimoku|O2 solo largos", {"dias": 10, "delta_sharpe": 0.0, "caida_base": 0.021916178968034217, "caida_var": 0.03073474802422349, "ret_base": -0.0035661661296341185, "ret_var": -0.03073474802422349, "p_boot": null}], ["S02 Ichimoku|O3 tama\u00f1o por volatilidad", {"dias": 10, "delta_sharpe": 0.0, "caida_base": 0.021916178968034217, "caida_var": 0.0165006851857864, "ret_base": -0.0035661661296341185, "ret_var": -0.002388520497693225, "p_boot": null}], ["S03 Bollinger + RSI (reversi\u00f3n)|O2 solo largos", {"dias": 10, "delta_sharpe": 0.0, "caida_base": 0.02314550224080769, "caida_var": 0.0, "ret_base": 0.020036096411532256, "ret_var": 0.00817678910011499, "p_boot": null}], ["S03 Bollinger + RSI (reversi\u00f3n)|O4 stop 3\u00d7ATR", {"dias": 10, "delta_sharpe": 0.0, "caida_base": 0.02314550224080769, "caida_var": 0.02382930038923925, "ret_base": 0.020036096411532256, "ret_var": 0.00527059403948793, "p_boot": null}]], "ultima_actualizacion": "2026-10-10 04:18:01.351761+00:00"}</t>
+          <t>{"n_pruebas": 75, "etapas": {"descartada (E1/E2)": 54, "E3 sombra": 21}, "adoptables": [], "top_forward": [["S03 Bollinger + RSI (reversi\u00f3n)|O2 solo largos", {"dias": 11, "delta_sharpe": 3.5537876160147945, "caida_base": 0.02314550224080769, "caida_var": 0.0, "ret_base": 0.030743633934825265, "ret_var": 0.01875983693281369, "p_boot": null}], ["S15 RSI14 + EMA200|O2 solo largos", {"dias": 11, "delta_sharpe": 3.4493534318148225, "caida_base": 0.047669256869431686, "caida_var": 0.02817103894115469, "ret_base": -0.027848657849687153, "ret_var": -0.007944628850053204, "p_boot": null}], ["S10 MACD + EMA200|O2 solo largos", {"dias": 11, "delta_sharpe": 2.3043402855521937, "caida_base": 0.026585235063741997, "caida_var": 0.01619791405258164, "ret_base": -0.007200591349225793, "ret_var": 0.0033935834350666827, "p_boot": null}], ["S09 Donchian 20/10|O2 solo largos", {"dias": 11, "delta_sharpe": 0.33110166095724747, "caida_base": 0.04810848142726609, "caida_var": 0.02817103894115469, "ret_base": -0.03770563290850304, "ret_var": -0.024359862351042594, "p_boot": null}], ["S08 Canal 20 por tercios|O3 tama\u00f1o por volatilidad", {"dias": 11, "delta_sharpe": 0.21231659685166981, "caida_base": 0.04008285523508037, "caida_var": 0.029523867371169077, "ret_base": -0.02857753563618093, "ret_var": -0.0204505814774959, "p_boot": null}]], "ultima_actualizacion": "2026-10-11 04:18:23.580833+00:00"}</t>
         </is>
       </c>
     </row>
@@ -703,7 +703,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I57"/>
+  <dimension ref="A1:I63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2392,6 +2392,204 @@
         <v>0.0041354473593871</v>
       </c>
       <c r="I57" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-10-09 04:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>983.5501954506448</v>
+      </c>
+      <c r="C58" t="n">
+        <v>0.003</v>
+      </c>
+      <c r="D58" t="n">
+        <v>82385.10000000001</v>
+      </c>
+      <c r="E58" t="n">
+        <v>0.2512889541817009</v>
+      </c>
+      <c r="F58" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G58" t="n">
+        <v>0.3718681508383357</v>
+      </c>
+      <c r="H58" t="n">
+        <v>0</v>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>OMITIDA_MIN_ORDEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-10-09 08:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>984.2334871625424</v>
+      </c>
+      <c r="C59" t="n">
+        <v>0.003</v>
+      </c>
+      <c r="D59" t="n">
+        <v>82617.2</v>
+      </c>
+      <c r="E59" t="n">
+        <v>0.2518219540716239</v>
+      </c>
+      <c r="F59" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G59" t="n">
+        <v>0.3730721904830374</v>
+      </c>
+      <c r="H59" t="n">
+        <v>0.0130082881021239</v>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>OMITIDA_MIN_ORDEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-10-09 12:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>985.9821871625426</v>
+      </c>
+      <c r="C60" t="n">
+        <v>0.003</v>
+      </c>
+      <c r="D60" t="n">
+        <v>83200.10000000001</v>
+      </c>
+      <c r="E60" t="n">
+        <v>0.2531488938134869</v>
+      </c>
+      <c r="F60" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G60" t="n">
+        <v>0.3732178305385936</v>
+      </c>
+      <c r="H60" t="n">
+        <v>0</v>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>OMITIDA_MIN_ORDEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-10-09 16:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>984.8966544112424</v>
+      </c>
+      <c r="C61" t="n">
+        <v>0.003</v>
+      </c>
+      <c r="D61" t="n">
+        <v>82839.39999999999</v>
+      </c>
+      <c r="E61" t="n">
+        <v>0.2523292153414418</v>
+      </c>
+      <c r="F61" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G61" t="n">
+        <v>0.3740154645146566</v>
+      </c>
+      <c r="H61" t="n">
+        <v>0.003432751300057</v>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>OMITIDA_MIN_ORDEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026-10-09 20:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>983.2937544112424</v>
+      </c>
+      <c r="C62" t="n">
+        <v>0.003</v>
+      </c>
+      <c r="D62" t="n">
+        <v>82305.10000000001</v>
+      </c>
+      <c r="E62" t="n">
+        <v>0.251110412216381</v>
+      </c>
+      <c r="F62" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G62" t="n">
+        <v>0.3741701015303192</v>
+      </c>
+      <c r="H62" t="n">
+        <v>0</v>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>OMITIDA_MIN_ORDEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-10-10 00:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>984.1010267234344</v>
+      </c>
+      <c r="C63" t="n">
+        <v>0.003</v>
+      </c>
+      <c r="D63" t="n">
+        <v>82578.5</v>
+      </c>
+      <c r="E63" t="n">
+        <v>0.2517378737270863</v>
+      </c>
+      <c r="F63" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G63" t="n">
+        <v>0.3752994372901202</v>
+      </c>
+      <c r="H63" t="n">
+        <v>0.0129276878079451</v>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>OMITIDA_MIN_ORDEN</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2691,10 +2889,10 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>-18.47210454935532</v>
+        <v>-15.89897327656547</v>
       </c>
       <c r="F2" t="n">
-        <v>-0.0184721045493553</v>
+        <v>-0.0158989732765654</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -2717,7 +2915,7 @@
         <v>0.875</v>
       </c>
       <c r="M2" t="n">
-        <v>9.166666666666666</v>
+        <v>10.16666666666667</v>
       </c>
     </row>
   </sheetData>
@@ -2828,10 +3026,10 @@
         <v>83579.11248</v>
       </c>
       <c r="G2" t="n">
-        <v>-14.97463907128256</v>
+        <v>-14.11692864701927</v>
       </c>
       <c r="H2" t="n">
-        <v>-0.0255953202847454</v>
+        <v>-0.0241292834129329</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -2839,7 +3037,7 @@
         </is>
       </c>
       <c r="J2" t="n">
-        <v>0.3941955773426058</v>
+        <v>0.4039851530793145</v>
       </c>
       <c r="K2" t="n">
         <v>0.0347417845660282</v>
@@ -2878,10 +3076,10 @@
         <v>83415.97986000001</v>
       </c>
       <c r="G3" t="n">
-        <v>-3.497465478072592</v>
+        <v>-1.782044629546009</v>
       </c>
       <c r="H3" t="n">
-        <v>-0.0209640016453832</v>
+        <v>-0.010681674138078</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
@@ -2889,7 +3087,7 @@
         </is>
       </c>
       <c r="J3" t="n">
-        <v>0.0040897782125769</v>
+        <v>0.0236689296859944</v>
       </c>
       <c r="K3" t="n">
         <v>0</v>
@@ -2964,22 +3162,22 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>-0.04809526346590653</v>
+        <v>-0.05593352757866366</v>
       </c>
       <c r="C2" t="n">
-        <v>0.05365393317356137</v>
+        <v>0.06450512282574605</v>
       </c>
       <c r="D2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F2" t="n">
-        <v>-14.7261078608289</v>
+        <v>-16.25893627154939</v>
       </c>
       <c r="G2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -2989,7 +3187,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>-0.003566166129633785</v>
+        <v>-0.01411122394983533</v>
       </c>
       <c r="C3" t="n">
         <v>0.04792737850644191</v>
@@ -2998,10 +3196,10 @@
         <v>3</v>
       </c>
       <c r="E3" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.8095873373892396</v>
+        <v>-3.010412212517539</v>
       </c>
       <c r="G3" t="n">
         <v>-1</v>
@@ -3014,7 +3212,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.02003609641153248</v>
+        <v>0.03074363393482571</v>
       </c>
       <c r="C4" t="n">
         <v>0.02560143416361205</v>
@@ -3023,10 +3221,10 @@
         <v>2</v>
       </c>
       <c r="E4" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F4" t="n">
-        <v>3.512173247518957</v>
+        <v>4.953362339748169</v>
       </c>
       <c r="G4" t="n">
         <v>1</v>
@@ -3039,19 +3237,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>-0.03067709352250236</v>
+        <v>-0.0409352418789749</v>
       </c>
       <c r="C5" t="n">
-        <v>0.04476296836728511</v>
+        <v>0.04809548795047969</v>
       </c>
       <c r="D5" t="n">
         <v>3</v>
       </c>
       <c r="E5" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F5" t="n">
-        <v>-5.683574990345989</v>
+        <v>-7.138471252338212</v>
       </c>
       <c r="G5" t="n">
         <v>-1</v>
@@ -3064,7 +3262,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>-0.029140530487063</v>
+        <v>-0.02181633521027726</v>
       </c>
       <c r="C6" t="n">
         <v>0.03768262617940443</v>
@@ -3073,13 +3271,13 @@
         <v>1</v>
       </c>
       <c r="E6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F6" t="n">
-        <v>-8.625102163836981</v>
+        <v>-5.464156619515538</v>
       </c>
       <c r="G6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -3089,7 +3287,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.02353863959080038</v>
+        <v>0.01270673709129166</v>
       </c>
       <c r="C7" t="n">
         <v>0.02757304106709146</v>
@@ -3098,10 +3296,10 @@
         <v>3</v>
       </c>
       <c r="E7" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F7" t="n">
-        <v>4.427907875174454</v>
+        <v>2.183788367764555</v>
       </c>
       <c r="G7" t="n">
         <v>-1</v>
@@ -3123,10 +3321,10 @@
         <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F8" t="n">
-        <v>0.234959276271921</v>
+        <v>0.2251517559894329</v>
       </c>
       <c r="G8" t="n">
         <v>0</v>
@@ -3139,22 +3337,22 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>-0.01317587620815053</v>
+        <v>-0.02857753563618026</v>
       </c>
       <c r="C9" t="n">
         <v>0.04396853436821047</v>
       </c>
       <c r="D9" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E9" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F9" t="n">
-        <v>-2.361791904094518</v>
+        <v>-4.601283393613085</v>
       </c>
       <c r="G9" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -3164,7 +3362,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>-0.02741294068242006</v>
+        <v>-0.03770563290850304</v>
       </c>
       <c r="C10" t="n">
         <v>0.05734111465474367</v>
@@ -3173,10 +3371,10 @@
         <v>3</v>
       </c>
       <c r="E10" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F10" t="n">
-        <v>-3.227394718133688</v>
+        <v>-4.267600760326958</v>
       </c>
       <c r="G10" t="n">
         <v>-1</v>
@@ -3189,22 +3387,22 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>-0.00330990881872717</v>
+        <v>-0.007200591349226015</v>
       </c>
       <c r="C11" t="n">
-        <v>0.03104399267694202</v>
+        <v>0.03797186285349852</v>
       </c>
       <c r="D11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E11" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F11" t="n">
-        <v>-0.6647363374726754</v>
+        <v>-1.457062100812373</v>
       </c>
       <c r="G11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
@@ -3214,7 +3412,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>-0.01413907664048075</v>
+        <v>-0.02457224348621423</v>
       </c>
       <c r="C12" t="n">
         <v>0.04447571020367225</v>
@@ -3223,10 +3421,10 @@
         <v>3</v>
       </c>
       <c r="E12" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F12" t="n">
-        <v>-1.944771278581969</v>
+        <v>-3.250997968322616</v>
       </c>
       <c r="G12" t="n">
         <v>-1</v>
@@ -3239,19 +3437,19 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>-0.02882819959249816</v>
+        <v>-0.03910591441965128</v>
       </c>
       <c r="C13" t="n">
-        <v>0.0318579706938229</v>
+        <v>0.04898319473768253</v>
       </c>
       <c r="D13" t="n">
         <v>5</v>
       </c>
       <c r="E13" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F13" t="n">
-        <v>-10.90069230266726</v>
+        <v>-12.85118271162761</v>
       </c>
       <c r="G13" t="n">
         <v>-1</v>
@@ -3273,10 +3471,10 @@
         <v>2</v>
       </c>
       <c r="E14" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F14" t="n">
-        <v>-1.191511098194244</v>
+        <v>-1.14156029321623</v>
       </c>
       <c r="G14" t="n">
         <v>0</v>
@@ -3289,7 +3487,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>-0.02350746917822688</v>
+        <v>-0.01325701779540533</v>
       </c>
       <c r="C15" t="n">
         <v>0.06348138346903642</v>
@@ -3298,10 +3496,10 @@
         <v>1</v>
       </c>
       <c r="E15" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F15" t="n">
-        <v>-3.142693006790305</v>
+        <v>-1.564867524079307</v>
       </c>
       <c r="G15" t="n">
         <v>1</v>
@@ -3314,19 +3512,19 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>-0.01745053550364284</v>
+        <v>-0.02784865784968726</v>
       </c>
       <c r="C16" t="n">
-        <v>0.03775837444115016</v>
+        <v>0.05477922770772337</v>
       </c>
       <c r="D16" t="n">
         <v>2</v>
       </c>
       <c r="E16" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F16" t="n">
-        <v>-3.278336021824348</v>
+        <v>-4.89008477566683</v>
       </c>
       <c r="G16" t="n">
         <v>-1</v>
@@ -3391,130 +3589,130 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>S01 Parabolic SAR + EMA200|O3 tamaño por volatilidad</t>
+          <t>S03 Bollinger + RSI (reversión)|O2 solo largos</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C2" t="n">
+        <v>3.553787616014795</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.02314550224080769</v>
+      </c>
+      <c r="E2" t="n">
         <v>0</v>
       </c>
-      <c r="D2" t="n">
-        <v>0.04806307582208469</v>
-      </c>
-      <c r="E2" t="n">
-        <v>0.03588632361481847</v>
-      </c>
       <c r="F2" t="n">
-        <v>-0.04809526346590665</v>
+        <v>0.03074363393482527</v>
       </c>
       <c r="G2" t="n">
-        <v>-0.03590909767315043</v>
+        <v>0.01875983693281369</v>
       </c>
       <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>S02 Ichimoku|O2 solo largos</t>
+          <t>S15 RSI14 + EMA200|O2 solo largos</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C3" t="n">
-        <v>0</v>
+        <v>3.449353431814822</v>
       </c>
       <c r="D3" t="n">
-        <v>0.02191617896803422</v>
+        <v>0.04766925686943169</v>
       </c>
       <c r="E3" t="n">
-        <v>0.03073474802422349</v>
+        <v>0.02817103894115469</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.003566166129634118</v>
+        <v>-0.02784865784968715</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.03073474802422349</v>
+        <v>-0.007944628850053204</v>
       </c>
       <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>S02 Ichimoku|O3 tamaño por volatilidad</t>
+          <t>S10 MACD + EMA200|O2 solo largos</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C4" t="n">
-        <v>0</v>
+        <v>2.304340285552194</v>
       </c>
       <c r="D4" t="n">
-        <v>0.02191617896803422</v>
+        <v>0.026585235063742</v>
       </c>
       <c r="E4" t="n">
-        <v>0.0165006851857864</v>
+        <v>0.01619791405258164</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.003566166129634118</v>
+        <v>-0.007200591349225793</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.002388520497693225</v>
+        <v>0.003393583435066683</v>
       </c>
       <c r="H4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>S03 Bollinger + RSI (reversión)|O2 solo largos</t>
+          <t>S09 Donchian 20/10|O2 solo largos</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C5" t="n">
-        <v>0</v>
+        <v>0.3311016609572475</v>
       </c>
       <c r="D5" t="n">
-        <v>0.02314550224080769</v>
+        <v>0.04810848142726609</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>0.02817103894115469</v>
       </c>
       <c r="F5" t="n">
-        <v>0.02003609641153226</v>
+        <v>-0.03770563290850304</v>
       </c>
       <c r="G5" t="n">
-        <v>0.008176789100114989</v>
+        <v>-0.02435986235104259</v>
       </c>
       <c r="H5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>S03 Bollinger + RSI (reversión)|O4 stop 3×ATR</t>
+          <t>S08 Canal 20 por tercios|O3 tamaño por volatilidad</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C6" t="n">
-        <v>0</v>
+        <v>0.2123165968516698</v>
       </c>
       <c r="D6" t="n">
-        <v>0.02314550224080769</v>
+        <v>0.04008285523508037</v>
       </c>
       <c r="E6" t="n">
-        <v>0.02382930038923925</v>
+        <v>0.02952386737116908</v>
       </c>
       <c r="F6" t="n">
-        <v>0.02003609641153226</v>
+        <v>-0.02857753563618093</v>
       </c>
       <c r="G6" t="n">
-        <v>0.00527059403948793</v>
+        <v>-0.0204505814774959</v>
       </c>
       <c r="H6" t="inlineStr"/>
     </row>

</xml_diff>